<commit_message>
update: 1. add new members
</commit_message>
<xml_diff>
--- a/process_avatar/final.xlsx
+++ b/process_avatar/final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SJTU\X-LANCE\宣传委员\xlance.github.io\process_avatar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7E4711-24F3-49B8-B89B-5FFC01FED619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1A2496-B6E7-4D8D-A06C-54BFC45B3733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-16840" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="827">
   <si>
     <t>name</t>
   </si>
@@ -709,36 +709,36 @@
     <t>/assets/img/members/student/许洪深.jpg</t>
   </si>
   <si>
+    <t>李杰宇</t>
+  </si>
+  <si>
+    <t>Jieyu Li</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/李杰宇.jpg</t>
+  </si>
+  <si>
+    <t>陈星宇</t>
+  </si>
+  <si>
+    <t>Xingyu Chen</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/陈星宇.jpg</t>
+  </si>
+  <si>
+    <t>马达</t>
+  </si>
+  <si>
+    <t>Da Ma</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/马达.jpg</t>
+  </si>
+  <si>
     <t>在读</t>
   </si>
   <si>
-    <t>李杰宇</t>
-  </si>
-  <si>
-    <t>Jieyu Li</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/李杰宇.jpg</t>
-  </si>
-  <si>
-    <t>陈星宇</t>
-  </si>
-  <si>
-    <t>Xingyu Chen</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/陈星宇.jpg</t>
-  </si>
-  <si>
-    <t>马达</t>
-  </si>
-  <si>
-    <t>Da Ma</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/马达.jpg</t>
-  </si>
-  <si>
     <t>吕波尔</t>
   </si>
   <si>
@@ -1129,6 +1129,9 @@
     <t>/assets/img/members/student/朱梓臣.jpg</t>
   </si>
   <si>
+    <t>JamesZhutheThird.github.io</t>
+  </si>
+  <si>
     <t>罗嘉鸣</t>
   </si>
   <si>
@@ -1315,6 +1318,9 @@
     <t>Senyu Han</t>
   </si>
   <si>
+    <t>UMP</t>
+  </si>
+  <si>
     <t>/assets/img/members/student/韩森宇.jpg</t>
   </si>
   <si>
@@ -1507,6 +1513,9 @@
     <t>/assets/img/members/student/刘丁烨.jpg</t>
   </si>
   <si>
+    <t>/assets/img/members/student/陈博_2.jpg</t>
+  </si>
+  <si>
     <t>李梓源</t>
   </si>
   <si>
@@ -1756,7 +1765,10 @@
     <t>Yushen Chen</t>
   </si>
   <si>
-    <t>/assets/img/members/student/陈禹伸.jpg</t>
+    <t>/assets/img/members/student/陈禹伸_2.jpg</t>
+  </si>
+  <si>
+    <t>github.com/SWivid</t>
   </si>
   <si>
     <t>迟佳颖</t>
@@ -1912,7 +1924,10 @@
     <t>Rui Xie</t>
   </si>
   <si>
-    <t>/assets/img/members/student/谢睿.jpg</t>
+    <t>/assets/img/members/student/谢睿_2.jpg</t>
+  </si>
+  <si>
+    <t>sharryxr.github.io</t>
   </si>
   <si>
     <t>徐瑞阳</t>
@@ -2008,7 +2023,7 @@
     <t>Zhangyi Kang</t>
   </si>
   <si>
-    <t>/assets/img/members/student/康张奕.jpg</t>
+    <t>/assets/img/members/student/康张奕_2.jpg</t>
   </si>
   <si>
     <t>刘筠彤</t>
@@ -2047,6 +2062,9 @@
     <t>/assets/img/members/student/马英梓.jpg</t>
   </si>
   <si>
+    <t>gray311.github.io</t>
+  </si>
+  <si>
     <t>涂文明</t>
   </si>
   <si>
@@ -2233,7 +2251,10 @@
     <t>Pengchao Feng</t>
   </si>
   <si>
-    <t>/assets/img/members/student/凤鹏超.jpg</t>
+    <t>/assets/img/members/student/凤鹏超_2.jpg</t>
+  </si>
+  <si>
+    <t>the-bird-f.github.io</t>
   </si>
   <si>
     <t>李亚霖</t>
@@ -2242,7 +2263,7 @@
     <t>Yalin Li</t>
   </si>
   <si>
-    <t>/assets/img/members/student/李亚霖.jpg</t>
+    <t>/assets/img/members/student/李亚霖_2.jpg</t>
   </si>
   <si>
     <t>张志龙</t>
@@ -2308,76 +2329,180 @@
     <t>/assets/img/members/student/李希泉.jpg</t>
   </si>
   <si>
+    <t>朱明瑄</t>
+  </si>
+  <si>
+    <t>Mingxuan Zhu</t>
+  </si>
+  <si>
+    <t>郑时捷</t>
+  </si>
+  <si>
+    <t>Shijie Zheng</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/郑时捷.jpg</t>
+  </si>
+  <si>
+    <t>张昊天</t>
+  </si>
+  <si>
+    <t>Haotian Zhang</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/张昊天.jpg</t>
+  </si>
+  <si>
+    <t>秦昊楠</t>
+  </si>
+  <si>
+    <t>Haonan Qin</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/秦昊楠.jpg</t>
+  </si>
+  <si>
+    <t>邢笑宇</t>
+  </si>
+  <si>
+    <t>Xiaoyu Xing</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/邢笑宇.jpg</t>
+  </si>
+  <si>
+    <t>王宇飞</t>
+  </si>
+  <si>
+    <t>Yufei Wang</t>
+  </si>
+  <si>
+    <t>霍彦儒</t>
+  </si>
+  <si>
+    <t>Yanru Huo</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/霍彦儒.jpg</t>
+  </si>
+  <si>
+    <t>岑智瀚</t>
+  </si>
+  <si>
+    <t>Zhihan Cen</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/岑智瀚.jpg</t>
+  </si>
+  <si>
+    <t>李昊</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/李昊.jpg</t>
+  </si>
+  <si>
+    <t>蒋铎鸣</t>
+  </si>
+  <si>
+    <t>Duoming Jiang</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/蒋铎鸣.jpg</t>
+  </si>
+  <si>
+    <t>李雨桐</t>
+  </si>
+  <si>
+    <t>Yutong Li</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/李雨桐.jpg</t>
+  </si>
+  <si>
+    <t>钱志恒</t>
+  </si>
+  <si>
+    <t>Zhiheng Qian</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/钱志恒.jpg</t>
+  </si>
+  <si>
+    <t>徐日晞</t>
+  </si>
+  <si>
+    <t>Rixi Xu</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/徐日晞.jpg</t>
+  </si>
+  <si>
+    <t>王柏雯</t>
+  </si>
+  <si>
+    <t>Bowen Wang</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/王柏雯.jpg</t>
+  </si>
+  <si>
+    <t>张语珩</t>
+  </si>
+  <si>
+    <t>Yuheng Zhang</t>
+  </si>
+  <si>
+    <t>Zhuo Li</t>
+  </si>
+  <si>
+    <t>邹知颖</t>
+  </si>
+  <si>
+    <t>Zhiying Zou</t>
+  </si>
+  <si>
+    <t>张之逸</t>
+  </si>
+  <si>
+    <t>Zhiyi Zhang</t>
+  </si>
+  <si>
+    <t>曹博涵</t>
+  </si>
+  <si>
+    <t>Bohan Cao</t>
+  </si>
+  <si>
+    <t>缪庆亮</t>
+  </si>
+  <si>
+    <t>Qingliang Miao</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/缪庆亮.jpg</t>
+  </si>
+  <si>
+    <t>彭坤杨</t>
+  </si>
+  <si>
+    <t>Kunyang Peng</t>
+  </si>
+  <si>
+    <t>刘贝易</t>
+  </si>
+  <si>
+    <t>Beiyi Liu</t>
+  </si>
+  <si>
     <t>xiquan-li.github.io</t>
-  </si>
-  <si>
-    <t>朱明瑄</t>
-  </si>
-  <si>
-    <t>Mingxuan Zhu</t>
-  </si>
-  <si>
-    <t>郑时捷</t>
-  </si>
-  <si>
-    <t>Shijie Zheng</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/郑时捷.jpg</t>
-  </si>
-  <si>
-    <t>张昊天</t>
-  </si>
-  <si>
-    <t>Haotian Zhang</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/张昊天.jpg</t>
-  </si>
-  <si>
-    <t>秦昊楠</t>
-  </si>
-  <si>
-    <t>Haonan Qin</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/秦昊楠.jpg</t>
-  </si>
-  <si>
-    <t>邢笑宇</t>
-  </si>
-  <si>
-    <t>Xiaoyu Xing</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/邢笑宇.jpg</t>
-  </si>
-  <si>
-    <t>U</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>JamesZhutheThird.github.io</t>
+    <t>李卓</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>/assets/img/members/student/陈博_2.jpg</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>UM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>M</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>王宇飞</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Yufei Wang</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2749,10 +2874,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G285"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="58.796875" customWidth="1"/>
+    <col min="5" max="5" width="45.06640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -4560,10 +4685,10 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
+        <v>229</v>
+      </c>
+      <c r="B91" t="s">
         <v>230</v>
-      </c>
-      <c r="B91" t="s">
-        <v>231</v>
       </c>
       <c r="C91">
         <v>92</v>
@@ -4572,7 +4697,7 @@
         <v>21</v>
       </c>
       <c r="E91" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F91" t="s">
         <v>11</v>
@@ -4580,10 +4705,10 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
+        <v>232</v>
+      </c>
+      <c r="B92" t="s">
         <v>233</v>
-      </c>
-      <c r="B92" t="s">
-        <v>234</v>
       </c>
       <c r="C92">
         <v>93</v>
@@ -4592,7 +4717,7 @@
         <v>78</v>
       </c>
       <c r="E92" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F92" t="s">
         <v>11</v>
@@ -4600,10 +4725,10 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
+        <v>235</v>
+      </c>
+      <c r="B93" t="s">
         <v>236</v>
-      </c>
-      <c r="B93" t="s">
-        <v>237</v>
       </c>
       <c r="C93">
         <v>94</v>
@@ -4612,10 +4737,10 @@
         <v>78</v>
       </c>
       <c r="E93" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F93" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
@@ -4809,7 +4934,7 @@
         <v>104</v>
       </c>
       <c r="D103" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E103" t="s">
         <v>14</v>
@@ -4855,7 +4980,7 @@
         <v>267</v>
       </c>
       <c r="F105" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
@@ -4875,7 +5000,7 @@
         <v>270</v>
       </c>
       <c r="F106" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.3">
@@ -4975,7 +5100,7 @@
         <v>285</v>
       </c>
       <c r="F111" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G111" t="s">
         <v>286</v>
@@ -5338,7 +5463,7 @@
         <v>328</v>
       </c>
       <c r="F129" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.3">
@@ -5478,7 +5603,7 @@
         <v>348</v>
       </c>
       <c r="F136" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.3">
@@ -5498,7 +5623,7 @@
         <v>351</v>
       </c>
       <c r="F137" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.3">
@@ -5538,7 +5663,7 @@
         <v>356</v>
       </c>
       <c r="F139" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.3">
@@ -5558,7 +5683,7 @@
         <v>359</v>
       </c>
       <c r="F140" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.3">
@@ -5578,7 +5703,7 @@
         <v>362</v>
       </c>
       <c r="F141" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.3">
@@ -5598,7 +5723,7 @@
         <v>365</v>
       </c>
       <c r="F142" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.3">
@@ -5618,18 +5743,18 @@
         <v>368</v>
       </c>
       <c r="F143" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G143" t="s">
-        <v>778</v>
+        <v>369</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B144" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C144">
         <v>147</v>
@@ -5638,18 +5763,18 @@
         <v>53</v>
       </c>
       <c r="E144" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F144" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B145" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C145">
         <v>148</v>
@@ -5658,7 +5783,7 @@
         <v>17</v>
       </c>
       <c r="E145" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F145" t="s">
         <v>11</v>
@@ -5666,10 +5791,10 @@
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B146" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C146">
         <v>149</v>
@@ -5678,7 +5803,7 @@
         <v>17</v>
       </c>
       <c r="E146" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F146" t="s">
         <v>11</v>
@@ -5686,10 +5811,10 @@
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B147" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C147">
         <v>150</v>
@@ -5698,18 +5823,18 @@
         <v>53</v>
       </c>
       <c r="E147" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F147" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B148" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C148">
         <v>151</v>
@@ -5718,18 +5843,18 @@
         <v>53</v>
       </c>
       <c r="E148" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F148" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B149" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C149">
         <v>152</v>
@@ -5741,15 +5866,15 @@
         <v>14</v>
       </c>
       <c r="F149" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B150" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C150">
         <v>153</v>
@@ -5758,18 +5883,18 @@
         <v>53</v>
       </c>
       <c r="E150" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F150" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B151" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C151">
         <v>154</v>
@@ -5778,7 +5903,7 @@
         <v>17</v>
       </c>
       <c r="E151" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F151" t="s">
         <v>11</v>
@@ -5786,10 +5911,10 @@
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B152" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C152">
         <v>155</v>
@@ -5798,7 +5923,7 @@
         <v>17</v>
       </c>
       <c r="E152" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F152" t="s">
         <v>11</v>
@@ -5806,10 +5931,10 @@
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B153" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C153">
         <v>156</v>
@@ -5818,18 +5943,18 @@
         <v>17</v>
       </c>
       <c r="E153" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F153" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B154" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C154">
         <v>157</v>
@@ -5838,18 +5963,18 @@
         <v>21</v>
       </c>
       <c r="E154" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F154" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B155" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C155">
         <v>158</v>
@@ -5858,21 +5983,21 @@
         <v>43</v>
       </c>
       <c r="E155" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F155" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G155" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B156" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C156">
         <v>159</v>
@@ -5881,18 +6006,18 @@
         <v>17</v>
       </c>
       <c r="E156" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F156" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B157" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C157">
         <v>160</v>
@@ -5901,18 +6026,18 @@
         <v>53</v>
       </c>
       <c r="E157" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F157" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B158" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C158">
         <v>161</v>
@@ -5921,18 +6046,18 @@
         <v>17</v>
       </c>
       <c r="E158" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F158" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B159" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C159">
         <v>162</v>
@@ -5941,38 +6066,38 @@
         <v>17</v>
       </c>
       <c r="E159" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F159" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B160" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C160">
         <v>163</v>
       </c>
       <c r="D160" t="s">
-        <v>781</v>
+        <v>78</v>
       </c>
       <c r="E160" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F160" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B161" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C161">
         <v>164</v>
@@ -5981,18 +6106,18 @@
         <v>53</v>
       </c>
       <c r="E161" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F161" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B162" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C162">
         <v>165</v>
@@ -6001,7 +6126,7 @@
         <v>17</v>
       </c>
       <c r="E162" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F162" t="s">
         <v>11</v>
@@ -6009,10 +6134,10 @@
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B163" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C163">
         <v>166</v>
@@ -6021,38 +6146,38 @@
         <v>53</v>
       </c>
       <c r="E163" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F163" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B164" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C164">
         <v>167</v>
       </c>
       <c r="D164" t="s">
-        <v>780</v>
+        <v>432</v>
       </c>
       <c r="E164" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F164" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B165" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C165">
         <v>168</v>
@@ -6061,7 +6186,7 @@
         <v>17</v>
       </c>
       <c r="E165" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="F165" t="s">
         <v>11</v>
@@ -6069,10 +6194,10 @@
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B166" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C166">
         <v>169</v>
@@ -6081,18 +6206,18 @@
         <v>43</v>
       </c>
       <c r="E166" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="F166" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B167" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C167">
         <v>170</v>
@@ -6101,7 +6226,7 @@
         <v>21</v>
       </c>
       <c r="E167" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F167" t="s">
         <v>11</v>
@@ -6109,10 +6234,10 @@
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B168" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C168">
         <v>171</v>
@@ -6121,21 +6246,21 @@
         <v>53</v>
       </c>
       <c r="E168" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="F168" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G168" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B169" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C169">
         <v>172</v>
@@ -6144,7 +6269,7 @@
         <v>17</v>
       </c>
       <c r="E169" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="F169" t="s">
         <v>11</v>
@@ -6152,10 +6277,10 @@
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B170" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C170">
         <v>173</v>
@@ -6164,38 +6289,38 @@
         <v>17</v>
       </c>
       <c r="E170" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F170" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B171" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C171">
         <v>174</v>
       </c>
       <c r="D171" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="E171" t="s">
         <v>14</v>
       </c>
       <c r="F171" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B172" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C172">
         <v>175</v>
@@ -6204,18 +6329,18 @@
         <v>17</v>
       </c>
       <c r="E172" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="F172" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B173" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="C173">
         <v>176</v>
@@ -6224,7 +6349,7 @@
         <v>17</v>
       </c>
       <c r="E173" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F173" t="s">
         <v>11</v>
@@ -6232,10 +6357,10 @@
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B174" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C174">
         <v>177</v>
@@ -6244,21 +6369,21 @@
         <v>43</v>
       </c>
       <c r="E174" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F174" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G174" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B175" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="C175">
         <v>178</v>
@@ -6267,21 +6392,21 @@
         <v>17</v>
       </c>
       <c r="E175" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F175" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G175" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B176" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="C176">
         <v>179</v>
@@ -6290,7 +6415,7 @@
         <v>17</v>
       </c>
       <c r="E176" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="F176" t="s">
         <v>11</v>
@@ -6298,10 +6423,10 @@
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B177" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C177">
         <v>180</v>
@@ -6318,10 +6443,10 @@
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B178" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C178">
         <v>181</v>
@@ -6338,10 +6463,10 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B179" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C179">
         <v>182</v>
@@ -6350,7 +6475,7 @@
         <v>17</v>
       </c>
       <c r="E179" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="F179" t="s">
         <v>11</v>
@@ -6358,10 +6483,10 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B180" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="C180">
         <v>183</v>
@@ -6370,18 +6495,18 @@
         <v>53</v>
       </c>
       <c r="E180" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="F180" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B181" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C181">
         <v>184</v>
@@ -6390,7 +6515,7 @@
         <v>43</v>
       </c>
       <c r="E181" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F181" t="s">
         <v>11</v>
@@ -6398,10 +6523,10 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B182" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C182">
         <v>185</v>
@@ -6410,18 +6535,18 @@
         <v>37</v>
       </c>
       <c r="E182" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="F182" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B183" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="C183">
         <v>186</v>
@@ -6430,18 +6555,18 @@
         <v>21</v>
       </c>
       <c r="E183" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F183" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B184" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C184">
         <v>187</v>
@@ -6450,18 +6575,18 @@
         <v>21</v>
       </c>
       <c r="E184" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="F184" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B185" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C185">
         <v>189</v>
@@ -6470,10 +6595,10 @@
         <v>17</v>
       </c>
       <c r="E185" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="F185" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
@@ -6490,18 +6615,18 @@
         <v>53</v>
       </c>
       <c r="E186" t="s">
-        <v>779</v>
+        <v>497</v>
       </c>
       <c r="F186" t="s">
-        <v>11</v>
+        <v>238</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B187" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="C187">
         <v>191</v>
@@ -6510,7 +6635,7 @@
         <v>9</v>
       </c>
       <c r="E187" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="F187" t="s">
         <v>11</v>
@@ -6518,10 +6643,10 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B188" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="C188">
         <v>192</v>
@@ -6530,18 +6655,18 @@
         <v>43</v>
       </c>
       <c r="E188" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="F188" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="B189" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="C189">
         <v>193</v>
@@ -6550,18 +6675,18 @@
         <v>21</v>
       </c>
       <c r="E189" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F189" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B190" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="C190">
         <v>194</v>
@@ -6570,18 +6695,18 @@
         <v>21</v>
       </c>
       <c r="E190" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F190" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="B191" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="C191">
         <v>195</v>
@@ -6590,18 +6715,18 @@
         <v>21</v>
       </c>
       <c r="E191" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="F191" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B192" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="C192">
         <v>196</v>
@@ -6618,10 +6743,10 @@
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B193" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C193">
         <v>197</v>
@@ -6630,18 +6755,18 @@
         <v>21</v>
       </c>
       <c r="E193" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="F193" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="B194" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="C194">
         <v>198</v>
@@ -6650,18 +6775,18 @@
         <v>17</v>
       </c>
       <c r="E194" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="F194" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B195" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C195">
         <v>199</v>
@@ -6678,10 +6803,10 @@
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B196" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="C196">
         <v>200</v>
@@ -6690,18 +6815,18 @@
         <v>43</v>
       </c>
       <c r="E196" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="F196" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="B197" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="C197">
         <v>202</v>
@@ -6710,18 +6835,18 @@
         <v>43</v>
       </c>
       <c r="E197" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="F197" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B198" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="C198">
         <v>203</v>
@@ -6730,18 +6855,18 @@
         <v>53</v>
       </c>
       <c r="E198" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="F198" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="B199" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="C199">
         <v>204</v>
@@ -6750,18 +6875,18 @@
         <v>21</v>
       </c>
       <c r="E199" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="F199" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B200" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C200">
         <v>205</v>
@@ -6770,18 +6895,18 @@
         <v>53</v>
       </c>
       <c r="E200" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="F200" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="B201" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="C201">
         <v>206</v>
@@ -6790,18 +6915,18 @@
         <v>43</v>
       </c>
       <c r="E201" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="F201" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="B202" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="C202">
         <v>208</v>
@@ -6810,18 +6935,18 @@
         <v>17</v>
       </c>
       <c r="E202" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="F202" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="B203" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C203">
         <v>209</v>
@@ -6830,18 +6955,18 @@
         <v>53</v>
       </c>
       <c r="E203" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="F203" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B204" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C204">
         <v>210</v>
@@ -6850,18 +6975,18 @@
         <v>43</v>
       </c>
       <c r="E204" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="F204" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="B205" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="C205">
         <v>213</v>
@@ -6870,18 +6995,18 @@
         <v>53</v>
       </c>
       <c r="E205" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="F205" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="B206" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C206">
         <v>214</v>
@@ -6890,18 +7015,18 @@
         <v>21</v>
       </c>
       <c r="E206" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="F206" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B207" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C207">
         <v>215</v>
@@ -6910,38 +7035,38 @@
         <v>21</v>
       </c>
       <c r="E207" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="F207" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B208" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C208">
         <v>216</v>
       </c>
       <c r="D208" t="s">
-        <v>21</v>
+        <v>826</v>
       </c>
       <c r="E208" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="F208" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B209" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C209">
         <v>217</v>
@@ -6950,18 +7075,18 @@
         <v>17</v>
       </c>
       <c r="E209" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="F209" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B210" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="C210">
         <v>218</v>
@@ -6970,18 +7095,18 @@
         <v>53</v>
       </c>
       <c r="E210" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="F210" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B211" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="C211">
         <v>219</v>
@@ -6990,35 +7115,35 @@
         <v>21</v>
       </c>
       <c r="E211" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="F211" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="212" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="B212" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="D212" t="s">
         <v>9</v>
       </c>
       <c r="E212" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="F212" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B213" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D213" t="s">
         <v>9</v>
@@ -7027,49 +7152,55 @@
         <v>14</v>
       </c>
       <c r="F213" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B214" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="D214" t="s">
         <v>21</v>
       </c>
       <c r="E214" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="F214" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B215" t="s">
-        <v>577</v>
+        <v>580</v>
+      </c>
+      <c r="C215">
+        <v>231</v>
       </c>
       <c r="D215" t="s">
-        <v>78</v>
+        <v>432</v>
       </c>
       <c r="E215" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="F215" t="s">
-        <v>229</v>
+        <v>238</v>
+      </c>
+      <c r="G215" t="s">
+        <v>582</v>
       </c>
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B216" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="D216" t="s">
         <v>9</v>
@@ -7078,49 +7209,49 @@
         <v>14</v>
       </c>
       <c r="F216" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="B217" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="D217" t="s">
         <v>9</v>
       </c>
       <c r="E217" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="F217" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="B218" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="D218" t="s">
         <v>21</v>
       </c>
       <c r="E218" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="F218" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="B219" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="D219" t="s">
         <v>21</v>
@@ -7134,30 +7265,33 @@
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="B220" t="s">
-        <v>590</v>
+        <v>594</v>
+      </c>
+      <c r="C220">
+        <v>227</v>
       </c>
       <c r="D220" t="s">
-        <v>777</v>
+        <v>9</v>
       </c>
       <c r="E220" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="F220" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G220" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="B221" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="D221" t="s">
         <v>9</v>
@@ -7166,15 +7300,15 @@
         <v>14</v>
       </c>
       <c r="F221" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="B222" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="D222" t="s">
         <v>21</v>
@@ -7183,32 +7317,32 @@
         <v>14</v>
       </c>
       <c r="F222" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="B223" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="D223" t="s">
         <v>9</v>
       </c>
       <c r="E223" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="F223" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="B224" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="D224" t="s">
         <v>9</v>
@@ -7217,15 +7351,15 @@
         <v>14</v>
       </c>
       <c r="F224" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="B225" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="C225">
         <v>212</v>
@@ -7234,44 +7368,44 @@
         <v>43</v>
       </c>
       <c r="E225" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="F225" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G225" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="B226" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="D226" t="s">
         <v>21</v>
       </c>
       <c r="E226" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="F226" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="B227" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="D227" t="s">
         <v>9</v>
       </c>
       <c r="E227" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="F227" t="s">
         <v>11</v>
@@ -7279,10 +7413,10 @@
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="B228" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="D228" t="s">
         <v>9</v>
@@ -7291,72 +7425,72 @@
         <v>14</v>
       </c>
       <c r="F228" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="B229" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D229" t="s">
         <v>9</v>
       </c>
       <c r="E229" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="F229" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="B230" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="D230" t="s">
         <v>9</v>
       </c>
       <c r="E230" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="F230" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B231" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="D231" t="s">
         <v>9</v>
       </c>
       <c r="E231" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="F231" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="B232" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="D232" t="s">
         <v>9</v>
       </c>
       <c r="E232" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="F232" t="s">
         <v>11</v>
@@ -7364,10 +7498,10 @@
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="B233" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="D233" t="s">
         <v>9</v>
@@ -7381,10 +7515,10 @@
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="B234" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="C234">
         <v>201</v>
@@ -7393,41 +7527,44 @@
         <v>43</v>
       </c>
       <c r="E234" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="F234" t="s">
-        <v>229</v>
+        <v>238</v>
+      </c>
+      <c r="G234" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="B235" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="D235" t="s">
         <v>9</v>
       </c>
       <c r="E235" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="F235" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="B236" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="D236" t="s">
         <v>9</v>
       </c>
       <c r="E236" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="F236" t="s">
         <v>11</v>
@@ -7435,33 +7572,33 @@
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="B237" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="D237" t="s">
         <v>9</v>
       </c>
       <c r="E237" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="F237" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="B238" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="D238" t="s">
         <v>9</v>
       </c>
       <c r="E238" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="F238" t="s">
         <v>11</v>
@@ -7469,16 +7606,16 @@
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="B239" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="D239" t="s">
         <v>9</v>
       </c>
       <c r="E239" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="F239" t="s">
         <v>11</v>
@@ -7486,10 +7623,10 @@
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="B240" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="D240" t="s">
         <v>9</v>
@@ -7498,15 +7635,15 @@
         <v>14</v>
       </c>
       <c r="F240" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="B241" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="D241" t="s">
         <v>9</v>
@@ -7515,15 +7652,15 @@
         <v>14</v>
       </c>
       <c r="F241" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="B242" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
       <c r="D242" t="s">
         <v>9</v>
@@ -7532,46 +7669,46 @@
         <v>14</v>
       </c>
       <c r="F242" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="B243" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="D243" t="s">
         <v>9</v>
       </c>
       <c r="E243" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="F243" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="B244" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="D244" t="s">
         <v>9</v>
       </c>
       <c r="E244" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="F244" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="B245" t="s">
         <v>290</v>
@@ -7580,103 +7717,109 @@
         <v>9</v>
       </c>
       <c r="E245" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="F245" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="B246" t="s">
-        <v>661</v>
+        <v>666</v>
+      </c>
+      <c r="C246">
+        <v>228</v>
       </c>
       <c r="D246" t="s">
         <v>21</v>
       </c>
       <c r="E246" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="F246" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="B247" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="D247" t="s">
         <v>9</v>
       </c>
       <c r="E247" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="F247" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="B248" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="D248" t="s">
         <v>9</v>
       </c>
       <c r="E248" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="F248" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="B249" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="D249" t="s">
         <v>9</v>
       </c>
       <c r="E249" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="F249" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="B250" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D250" t="s">
         <v>9</v>
       </c>
       <c r="E250" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="F250" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G250" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="B251" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="C251">
         <v>207</v>
@@ -7685,35 +7828,35 @@
         <v>53</v>
       </c>
       <c r="E251" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="F251" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="B252" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="D252" t="s">
         <v>17</v>
       </c>
       <c r="E252" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="F252" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="253" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="B253" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="C253">
         <v>211</v>
@@ -7722,205 +7865,208 @@
         <v>17</v>
       </c>
       <c r="E253" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="F253" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="B254" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="D254" t="s">
         <v>9</v>
       </c>
       <c r="E254" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="F254" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="255" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="B255" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D255" t="s">
         <v>53</v>
       </c>
       <c r="E255" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="F255" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="256" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="B256" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="D256" t="s">
         <v>9</v>
       </c>
       <c r="E256" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="F256" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="B257" t="s">
-        <v>694</v>
+        <v>700</v>
+      </c>
+      <c r="C257">
+        <v>230</v>
       </c>
       <c r="D257" t="s">
         <v>53</v>
       </c>
       <c r="E257" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="F257" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="B258" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="D258" t="s">
         <v>9</v>
       </c>
       <c r="E258" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="F258" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="B259" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="D259" t="s">
         <v>9</v>
       </c>
       <c r="E259" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="F259" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="B260" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="D260" t="s">
         <v>9</v>
       </c>
       <c r="E260" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="F260" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="B261" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="D261" t="s">
         <v>9</v>
       </c>
       <c r="E261" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="F261" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="B262" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="D262" t="s">
         <v>9</v>
       </c>
       <c r="E262" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="F262" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="B263" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="D263" t="s">
         <v>9</v>
       </c>
       <c r="E263" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="F263" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="B264" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="D264" t="s">
         <v>9</v>
       </c>
       <c r="E264" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="F264" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="B265" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="D265" t="s">
         <v>9</v>
@@ -7929,137 +8075,140 @@
         <v>14</v>
       </c>
       <c r="F265" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="B266" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="D266" t="s">
         <v>9</v>
       </c>
       <c r="E266" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="F266" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="B267" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="D267" t="s">
         <v>17</v>
       </c>
       <c r="E267" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="F267" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="B268" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="D268" t="s">
         <v>9</v>
       </c>
       <c r="E268" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="F268" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="B269" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="D269" t="s">
-        <v>777</v>
+        <v>9</v>
       </c>
       <c r="E269" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="F269" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G269" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
     </row>
     <row r="270" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B270" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="D270" t="s">
         <v>9</v>
       </c>
       <c r="E270" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="F270" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="271" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="B271" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="D271" t="s">
         <v>9</v>
       </c>
       <c r="E271" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="F271" t="s">
-        <v>229</v>
+        <v>238</v>
+      </c>
+      <c r="G271" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
       <c r="B272" t="s">
-        <v>739</v>
+        <v>746</v>
       </c>
       <c r="D272" t="s">
         <v>9</v>
       </c>
       <c r="E272" t="s">
-        <v>740</v>
+        <v>747</v>
       </c>
       <c r="F272" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
-        <v>741</v>
+        <v>748</v>
       </c>
       <c r="B273" t="s">
-        <v>742</v>
+        <v>749</v>
       </c>
       <c r="C273">
         <v>220</v>
@@ -8076,16 +8225,16 @@
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="B274" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="D274" t="s">
         <v>9</v>
       </c>
       <c r="E274" t="s">
-        <v>745</v>
+        <v>752</v>
       </c>
       <c r="F274" t="s">
         <v>11</v>
@@ -8093,27 +8242,27 @@
     </row>
     <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
-        <v>746</v>
+        <v>753</v>
       </c>
       <c r="B275" t="s">
-        <v>747</v>
+        <v>754</v>
       </c>
       <c r="D275" t="s">
         <v>9</v>
       </c>
       <c r="E275" t="s">
-        <v>748</v>
+        <v>755</v>
       </c>
       <c r="F275" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
-        <v>749</v>
+        <v>756</v>
       </c>
       <c r="B276" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="C276">
         <v>196</v>
@@ -8122,75 +8271,75 @@
         <v>17</v>
       </c>
       <c r="E276" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
       <c r="F276" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G276" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
-        <v>753</v>
+        <v>760</v>
       </c>
       <c r="B277" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="D277" t="s">
         <v>9</v>
       </c>
       <c r="E277" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
       <c r="F277" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
-        <v>756</v>
+        <v>763</v>
       </c>
       <c r="B278" t="s">
-        <v>757</v>
+        <v>764</v>
       </c>
       <c r="D278" t="s">
         <v>9</v>
       </c>
       <c r="E278" t="s">
-        <v>758</v>
+        <v>765</v>
       </c>
       <c r="F278" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
       <c r="B279" t="s">
-        <v>760</v>
+        <v>767</v>
       </c>
       <c r="D279" t="s">
         <v>21</v>
       </c>
       <c r="E279" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="F279" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G279" t="s">
-        <v>762</v>
+        <v>824</v>
       </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="B280" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="D280" t="s">
         <v>9</v>
@@ -8199,97 +8348,369 @@
         <v>14</v>
       </c>
       <c r="F280" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="B281" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="D281" t="s">
         <v>9</v>
       </c>
       <c r="E281" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="F281" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="B282" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="D282" t="s">
         <v>17</v>
       </c>
       <c r="E282" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="F282" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="B283" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="D283" t="s">
         <v>9</v>
       </c>
       <c r="E283" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="F283" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="B284" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="D284" t="s">
         <v>9</v>
       </c>
       <c r="E284" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="F284" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="B285" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="D285" t="s">
-        <v>781</v>
+        <v>17</v>
       </c>
       <c r="E285" t="s">
         <v>14</v>
       </c>
       <c r="F285" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A286" t="s">
+        <v>785</v>
+      </c>
+      <c r="B286" t="s">
+        <v>786</v>
+      </c>
+      <c r="D286" t="s">
+        <v>9</v>
+      </c>
+      <c r="E286" t="s">
+        <v>787</v>
+      </c>
+      <c r="F286" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A287" t="s">
+        <v>788</v>
+      </c>
+      <c r="B287" t="s">
+        <v>789</v>
+      </c>
+      <c r="D287" t="s">
+        <v>9</v>
+      </c>
+      <c r="E287" t="s">
+        <v>790</v>
+      </c>
+      <c r="F287" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A288" t="s">
+        <v>791</v>
+      </c>
+      <c r="B288" t="s">
+        <v>167</v>
+      </c>
+      <c r="D288" t="s">
+        <v>17</v>
+      </c>
+      <c r="E288" t="s">
+        <v>792</v>
+      </c>
+      <c r="F288" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="289" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A289" t="s">
+        <v>793</v>
+      </c>
+      <c r="B289" t="s">
+        <v>794</v>
+      </c>
+      <c r="D289" t="s">
+        <v>9</v>
+      </c>
+      <c r="E289" t="s">
+        <v>795</v>
+      </c>
+      <c r="F289" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A290" t="s">
+        <v>796</v>
+      </c>
+      <c r="B290" t="s">
+        <v>797</v>
+      </c>
+      <c r="D290" t="s">
+        <v>9</v>
+      </c>
+      <c r="E290" t="s">
+        <v>798</v>
+      </c>
+      <c r="F290" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="291" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A291" t="s">
+        <v>799</v>
+      </c>
+      <c r="B291" t="s">
+        <v>800</v>
+      </c>
+      <c r="D291" t="s">
+        <v>9</v>
+      </c>
+      <c r="E291" t="s">
+        <v>801</v>
+      </c>
+      <c r="F291" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="292" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A292" t="s">
+        <v>802</v>
+      </c>
+      <c r="B292" t="s">
+        <v>803</v>
+      </c>
+      <c r="D292" t="s">
+        <v>9</v>
+      </c>
+      <c r="E292" t="s">
+        <v>804</v>
+      </c>
+      <c r="F292" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="293" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A293" t="s">
+        <v>805</v>
+      </c>
+      <c r="B293" t="s">
+        <v>806</v>
+      </c>
+      <c r="D293" t="s">
+        <v>9</v>
+      </c>
+      <c r="E293" t="s">
+        <v>807</v>
+      </c>
+      <c r="F293" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A294" t="s">
+        <v>808</v>
+      </c>
+      <c r="B294" t="s">
+        <v>809</v>
+      </c>
+      <c r="D294" t="s">
+        <v>17</v>
+      </c>
+      <c r="E294" t="s">
+        <v>14</v>
+      </c>
+      <c r="F294" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A295" t="s">
+        <v>825</v>
+      </c>
+      <c r="B295" t="s">
+        <v>810</v>
+      </c>
+      <c r="D295" t="s">
+        <v>17</v>
+      </c>
+      <c r="E295" t="s">
+        <v>14</v>
+      </c>
+      <c r="F295" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A296" t="s">
+        <v>811</v>
+      </c>
+      <c r="B296" t="s">
+        <v>812</v>
+      </c>
+      <c r="D296" t="s">
+        <v>17</v>
+      </c>
+      <c r="E296" t="s">
+        <v>14</v>
+      </c>
+      <c r="F296" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A297" t="s">
+        <v>813</v>
+      </c>
+      <c r="B297" t="s">
+        <v>814</v>
+      </c>
+      <c r="D297" t="s">
+        <v>17</v>
+      </c>
+      <c r="E297" t="s">
+        <v>14</v>
+      </c>
+      <c r="F297" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="298" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A298" t="s">
+        <v>815</v>
+      </c>
+      <c r="B298" t="s">
+        <v>816</v>
+      </c>
+      <c r="D298" t="s">
+        <v>17</v>
+      </c>
+      <c r="E298" t="s">
+        <v>14</v>
+      </c>
+      <c r="F298" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="299" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A299" t="s">
+        <v>817</v>
+      </c>
+      <c r="B299" t="s">
+        <v>818</v>
+      </c>
+      <c r="D299" t="s">
+        <v>37</v>
+      </c>
+      <c r="E299" t="s">
+        <v>819</v>
+      </c>
+      <c r="F299" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="300" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A300" t="s">
+        <v>820</v>
+      </c>
+      <c r="B300" t="s">
+        <v>821</v>
+      </c>
+      <c r="D300" t="s">
+        <v>37</v>
+      </c>
+      <c r="E300" t="s">
+        <v>14</v>
+      </c>
+      <c r="F300" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="301" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A301" t="s">
+        <v>822</v>
+      </c>
+      <c r="B301" t="s">
+        <v>823</v>
+      </c>
+      <c r="D301" t="s">
+        <v>37</v>
+      </c>
+      <c r="E301" t="s">
+        <v>14</v>
+      </c>
+      <c r="F301" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Deploying to gh-pages from @ X-LANCE/x-lance.github.io@34bf097f8f7131f7c1144f8b63cd3bc2c5915e1b 🚀
</commit_message>
<xml_diff>
--- a/process_avatar/final.xlsx
+++ b/process_avatar/final.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SJTU\X-LANCE\宣传委员\xlance.github.io\process_avatar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B7E4711-24F3-49B8-B89B-5FFC01FED619}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1A2496-B6E7-4D8D-A06C-54BFC45B3733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-16840" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1438" uniqueCount="784">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1522" uniqueCount="827">
   <si>
     <t>name</t>
   </si>
@@ -709,36 +709,36 @@
     <t>/assets/img/members/student/许洪深.jpg</t>
   </si>
   <si>
+    <t>李杰宇</t>
+  </si>
+  <si>
+    <t>Jieyu Li</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/李杰宇.jpg</t>
+  </si>
+  <si>
+    <t>陈星宇</t>
+  </si>
+  <si>
+    <t>Xingyu Chen</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/陈星宇.jpg</t>
+  </si>
+  <si>
+    <t>马达</t>
+  </si>
+  <si>
+    <t>Da Ma</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/马达.jpg</t>
+  </si>
+  <si>
     <t>在读</t>
   </si>
   <si>
-    <t>李杰宇</t>
-  </si>
-  <si>
-    <t>Jieyu Li</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/李杰宇.jpg</t>
-  </si>
-  <si>
-    <t>陈星宇</t>
-  </si>
-  <si>
-    <t>Xingyu Chen</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/陈星宇.jpg</t>
-  </si>
-  <si>
-    <t>马达</t>
-  </si>
-  <si>
-    <t>Da Ma</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/马达.jpg</t>
-  </si>
-  <si>
     <t>吕波尔</t>
   </si>
   <si>
@@ -1129,6 +1129,9 @@
     <t>/assets/img/members/student/朱梓臣.jpg</t>
   </si>
   <si>
+    <t>JamesZhutheThird.github.io</t>
+  </si>
+  <si>
     <t>罗嘉鸣</t>
   </si>
   <si>
@@ -1315,6 +1318,9 @@
     <t>Senyu Han</t>
   </si>
   <si>
+    <t>UMP</t>
+  </si>
+  <si>
     <t>/assets/img/members/student/韩森宇.jpg</t>
   </si>
   <si>
@@ -1507,6 +1513,9 @@
     <t>/assets/img/members/student/刘丁烨.jpg</t>
   </si>
   <si>
+    <t>/assets/img/members/student/陈博_2.jpg</t>
+  </si>
+  <si>
     <t>李梓源</t>
   </si>
   <si>
@@ -1756,7 +1765,10 @@
     <t>Yushen Chen</t>
   </si>
   <si>
-    <t>/assets/img/members/student/陈禹伸.jpg</t>
+    <t>/assets/img/members/student/陈禹伸_2.jpg</t>
+  </si>
+  <si>
+    <t>github.com/SWivid</t>
   </si>
   <si>
     <t>迟佳颖</t>
@@ -1912,7 +1924,10 @@
     <t>Rui Xie</t>
   </si>
   <si>
-    <t>/assets/img/members/student/谢睿.jpg</t>
+    <t>/assets/img/members/student/谢睿_2.jpg</t>
+  </si>
+  <si>
+    <t>sharryxr.github.io</t>
   </si>
   <si>
     <t>徐瑞阳</t>
@@ -2008,7 +2023,7 @@
     <t>Zhangyi Kang</t>
   </si>
   <si>
-    <t>/assets/img/members/student/康张奕.jpg</t>
+    <t>/assets/img/members/student/康张奕_2.jpg</t>
   </si>
   <si>
     <t>刘筠彤</t>
@@ -2047,6 +2062,9 @@
     <t>/assets/img/members/student/马英梓.jpg</t>
   </si>
   <si>
+    <t>gray311.github.io</t>
+  </si>
+  <si>
     <t>涂文明</t>
   </si>
   <si>
@@ -2233,7 +2251,10 @@
     <t>Pengchao Feng</t>
   </si>
   <si>
-    <t>/assets/img/members/student/凤鹏超.jpg</t>
+    <t>/assets/img/members/student/凤鹏超_2.jpg</t>
+  </si>
+  <si>
+    <t>the-bird-f.github.io</t>
   </si>
   <si>
     <t>李亚霖</t>
@@ -2242,7 +2263,7 @@
     <t>Yalin Li</t>
   </si>
   <si>
-    <t>/assets/img/members/student/李亚霖.jpg</t>
+    <t>/assets/img/members/student/李亚霖_2.jpg</t>
   </si>
   <si>
     <t>张志龙</t>
@@ -2308,76 +2329,180 @@
     <t>/assets/img/members/student/李希泉.jpg</t>
   </si>
   <si>
+    <t>朱明瑄</t>
+  </si>
+  <si>
+    <t>Mingxuan Zhu</t>
+  </si>
+  <si>
+    <t>郑时捷</t>
+  </si>
+  <si>
+    <t>Shijie Zheng</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/郑时捷.jpg</t>
+  </si>
+  <si>
+    <t>张昊天</t>
+  </si>
+  <si>
+    <t>Haotian Zhang</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/张昊天.jpg</t>
+  </si>
+  <si>
+    <t>秦昊楠</t>
+  </si>
+  <si>
+    <t>Haonan Qin</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/秦昊楠.jpg</t>
+  </si>
+  <si>
+    <t>邢笑宇</t>
+  </si>
+  <si>
+    <t>Xiaoyu Xing</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/邢笑宇.jpg</t>
+  </si>
+  <si>
+    <t>王宇飞</t>
+  </si>
+  <si>
+    <t>Yufei Wang</t>
+  </si>
+  <si>
+    <t>霍彦儒</t>
+  </si>
+  <si>
+    <t>Yanru Huo</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/霍彦儒.jpg</t>
+  </si>
+  <si>
+    <t>岑智瀚</t>
+  </si>
+  <si>
+    <t>Zhihan Cen</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/岑智瀚.jpg</t>
+  </si>
+  <si>
+    <t>李昊</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/李昊.jpg</t>
+  </si>
+  <si>
+    <t>蒋铎鸣</t>
+  </si>
+  <si>
+    <t>Duoming Jiang</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/蒋铎鸣.jpg</t>
+  </si>
+  <si>
+    <t>李雨桐</t>
+  </si>
+  <si>
+    <t>Yutong Li</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/李雨桐.jpg</t>
+  </si>
+  <si>
+    <t>钱志恒</t>
+  </si>
+  <si>
+    <t>Zhiheng Qian</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/钱志恒.jpg</t>
+  </si>
+  <si>
+    <t>徐日晞</t>
+  </si>
+  <si>
+    <t>Rixi Xu</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/徐日晞.jpg</t>
+  </si>
+  <si>
+    <t>王柏雯</t>
+  </si>
+  <si>
+    <t>Bowen Wang</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/王柏雯.jpg</t>
+  </si>
+  <si>
+    <t>张语珩</t>
+  </si>
+  <si>
+    <t>Yuheng Zhang</t>
+  </si>
+  <si>
+    <t>Zhuo Li</t>
+  </si>
+  <si>
+    <t>邹知颖</t>
+  </si>
+  <si>
+    <t>Zhiying Zou</t>
+  </si>
+  <si>
+    <t>张之逸</t>
+  </si>
+  <si>
+    <t>Zhiyi Zhang</t>
+  </si>
+  <si>
+    <t>曹博涵</t>
+  </si>
+  <si>
+    <t>Bohan Cao</t>
+  </si>
+  <si>
+    <t>缪庆亮</t>
+  </si>
+  <si>
+    <t>Qingliang Miao</t>
+  </si>
+  <si>
+    <t>/assets/img/members/student/缪庆亮.jpg</t>
+  </si>
+  <si>
+    <t>彭坤杨</t>
+  </si>
+  <si>
+    <t>Kunyang Peng</t>
+  </si>
+  <si>
+    <t>刘贝易</t>
+  </si>
+  <si>
+    <t>Beiyi Liu</t>
+  </si>
+  <si>
     <t>xiquan-li.github.io</t>
-  </si>
-  <si>
-    <t>朱明瑄</t>
-  </si>
-  <si>
-    <t>Mingxuan Zhu</t>
-  </si>
-  <si>
-    <t>郑时捷</t>
-  </si>
-  <si>
-    <t>Shijie Zheng</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/郑时捷.jpg</t>
-  </si>
-  <si>
-    <t>张昊天</t>
-  </si>
-  <si>
-    <t>Haotian Zhang</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/张昊天.jpg</t>
-  </si>
-  <si>
-    <t>秦昊楠</t>
-  </si>
-  <si>
-    <t>Haonan Qin</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/秦昊楠.jpg</t>
-  </si>
-  <si>
-    <t>邢笑宇</t>
-  </si>
-  <si>
-    <t>Xiaoyu Xing</t>
-  </si>
-  <si>
-    <t>/assets/img/members/student/邢笑宇.jpg</t>
-  </si>
-  <si>
-    <t>U</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>JamesZhutheThird.github.io</t>
+    <t>李卓</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>/assets/img/members/student/陈博_2.jpg</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>UM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>M</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>王宇飞</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Yufei Wang</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -2749,10 +2874,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G285"/>
+  <dimension ref="A1:G301"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="5" max="5" width="58.796875" customWidth="1"/>
+    <col min="5" max="5" width="45.06640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -4560,10 +4685,10 @@
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
+        <v>229</v>
+      </c>
+      <c r="B91" t="s">
         <v>230</v>
-      </c>
-      <c r="B91" t="s">
-        <v>231</v>
       </c>
       <c r="C91">
         <v>92</v>
@@ -4572,7 +4697,7 @@
         <v>21</v>
       </c>
       <c r="E91" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="F91" t="s">
         <v>11</v>
@@ -4580,10 +4705,10 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
+        <v>232</v>
+      </c>
+      <c r="B92" t="s">
         <v>233</v>
-      </c>
-      <c r="B92" t="s">
-        <v>234</v>
       </c>
       <c r="C92">
         <v>93</v>
@@ -4592,7 +4717,7 @@
         <v>78</v>
       </c>
       <c r="E92" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F92" t="s">
         <v>11</v>
@@ -4600,10 +4725,10 @@
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
+        <v>235</v>
+      </c>
+      <c r="B93" t="s">
         <v>236</v>
-      </c>
-      <c r="B93" t="s">
-        <v>237</v>
       </c>
       <c r="C93">
         <v>94</v>
@@ -4612,10 +4737,10 @@
         <v>78</v>
       </c>
       <c r="E93" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F93" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
@@ -4809,7 +4934,7 @@
         <v>104</v>
       </c>
       <c r="D103" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E103" t="s">
         <v>14</v>
@@ -4855,7 +4980,7 @@
         <v>267</v>
       </c>
       <c r="F105" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
@@ -4875,7 +5000,7 @@
         <v>270</v>
       </c>
       <c r="F106" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.3">
@@ -4975,7 +5100,7 @@
         <v>285</v>
       </c>
       <c r="F111" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G111" t="s">
         <v>286</v>
@@ -5338,7 +5463,7 @@
         <v>328</v>
       </c>
       <c r="F129" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.3">
@@ -5478,7 +5603,7 @@
         <v>348</v>
       </c>
       <c r="F136" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.3">
@@ -5498,7 +5623,7 @@
         <v>351</v>
       </c>
       <c r="F137" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.3">
@@ -5538,7 +5663,7 @@
         <v>356</v>
       </c>
       <c r="F139" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.3">
@@ -5558,7 +5683,7 @@
         <v>359</v>
       </c>
       <c r="F140" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.3">
@@ -5578,7 +5703,7 @@
         <v>362</v>
       </c>
       <c r="F141" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.3">
@@ -5598,7 +5723,7 @@
         <v>365</v>
       </c>
       <c r="F142" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.3">
@@ -5618,18 +5743,18 @@
         <v>368</v>
       </c>
       <c r="F143" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G143" t="s">
-        <v>778</v>
+        <v>369</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B144" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C144">
         <v>147</v>
@@ -5638,18 +5763,18 @@
         <v>53</v>
       </c>
       <c r="E144" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F144" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B145" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C145">
         <v>148</v>
@@ -5658,7 +5783,7 @@
         <v>17</v>
       </c>
       <c r="E145" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="F145" t="s">
         <v>11</v>
@@ -5666,10 +5791,10 @@
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B146" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C146">
         <v>149</v>
@@ -5678,7 +5803,7 @@
         <v>17</v>
       </c>
       <c r="E146" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F146" t="s">
         <v>11</v>
@@ -5686,10 +5811,10 @@
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B147" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C147">
         <v>150</v>
@@ -5698,18 +5823,18 @@
         <v>53</v>
       </c>
       <c r="E147" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F147" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B148" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C148">
         <v>151</v>
@@ -5718,18 +5843,18 @@
         <v>53</v>
       </c>
       <c r="E148" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F148" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B149" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C149">
         <v>152</v>
@@ -5741,15 +5866,15 @@
         <v>14</v>
       </c>
       <c r="F149" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B150" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C150">
         <v>153</v>
@@ -5758,18 +5883,18 @@
         <v>53</v>
       </c>
       <c r="E150" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F150" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B151" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C151">
         <v>154</v>
@@ -5778,7 +5903,7 @@
         <v>17</v>
       </c>
       <c r="E151" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="F151" t="s">
         <v>11</v>
@@ -5786,10 +5911,10 @@
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B152" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C152">
         <v>155</v>
@@ -5798,7 +5923,7 @@
         <v>17</v>
       </c>
       <c r="E152" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F152" t="s">
         <v>11</v>
@@ -5806,10 +5931,10 @@
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B153" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C153">
         <v>156</v>
@@ -5818,18 +5943,18 @@
         <v>17</v>
       </c>
       <c r="E153" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F153" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B154" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C154">
         <v>157</v>
@@ -5838,18 +5963,18 @@
         <v>21</v>
       </c>
       <c r="E154" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F154" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B155" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C155">
         <v>158</v>
@@ -5858,21 +5983,21 @@
         <v>43</v>
       </c>
       <c r="E155" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F155" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G155" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="B156" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C156">
         <v>159</v>
@@ -5881,18 +6006,18 @@
         <v>17</v>
       </c>
       <c r="E156" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F156" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="B157" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="C157">
         <v>160</v>
@@ -5901,18 +6026,18 @@
         <v>53</v>
       </c>
       <c r="E157" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F157" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="B158" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="C158">
         <v>161</v>
@@ -5921,18 +6046,18 @@
         <v>17</v>
       </c>
       <c r="E158" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F158" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B159" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="C159">
         <v>162</v>
@@ -5941,38 +6066,38 @@
         <v>17</v>
       </c>
       <c r="E159" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="F159" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B160" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="C160">
         <v>163</v>
       </c>
       <c r="D160" t="s">
-        <v>781</v>
+        <v>78</v>
       </c>
       <c r="E160" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F160" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B161" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C161">
         <v>164</v>
@@ -5981,18 +6106,18 @@
         <v>53</v>
       </c>
       <c r="E161" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F161" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="B162" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="C162">
         <v>165</v>
@@ -6001,7 +6126,7 @@
         <v>17</v>
       </c>
       <c r="E162" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F162" t="s">
         <v>11</v>
@@ -6009,10 +6134,10 @@
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="B163" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="C163">
         <v>166</v>
@@ -6021,38 +6146,38 @@
         <v>53</v>
       </c>
       <c r="E163" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="F163" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="B164" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="C164">
         <v>167</v>
       </c>
       <c r="D164" t="s">
-        <v>780</v>
+        <v>432</v>
       </c>
       <c r="E164" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="F164" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B165" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C165">
         <v>168</v>
@@ -6061,7 +6186,7 @@
         <v>17</v>
       </c>
       <c r="E165" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="F165" t="s">
         <v>11</v>
@@ -6069,10 +6194,10 @@
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B166" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="C166">
         <v>169</v>
@@ -6081,18 +6206,18 @@
         <v>43</v>
       </c>
       <c r="E166" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="F166" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B167" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="C167">
         <v>170</v>
@@ -6101,7 +6226,7 @@
         <v>21</v>
       </c>
       <c r="E167" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F167" t="s">
         <v>11</v>
@@ -6109,10 +6234,10 @@
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B168" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="C168">
         <v>171</v>
@@ -6121,21 +6246,21 @@
         <v>53</v>
       </c>
       <c r="E168" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="F168" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G168" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B169" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="C169">
         <v>172</v>
@@ -6144,7 +6269,7 @@
         <v>17</v>
       </c>
       <c r="E169" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="F169" t="s">
         <v>11</v>
@@ -6152,10 +6277,10 @@
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B170" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C170">
         <v>173</v>
@@ -6164,38 +6289,38 @@
         <v>17</v>
       </c>
       <c r="E170" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F170" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B171" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="C171">
         <v>174</v>
       </c>
       <c r="D171" t="s">
-        <v>17</v>
+        <v>78</v>
       </c>
       <c r="E171" t="s">
         <v>14</v>
       </c>
       <c r="F171" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B172" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="C172">
         <v>175</v>
@@ -6204,18 +6329,18 @@
         <v>17</v>
       </c>
       <c r="E172" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="F172" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B173" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="C173">
         <v>176</v>
@@ -6224,7 +6349,7 @@
         <v>17</v>
       </c>
       <c r="E173" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F173" t="s">
         <v>11</v>
@@ -6232,10 +6357,10 @@
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B174" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="C174">
         <v>177</v>
@@ -6244,21 +6369,21 @@
         <v>43</v>
       </c>
       <c r="E174" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F174" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G174" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B175" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="C175">
         <v>178</v>
@@ -6267,21 +6392,21 @@
         <v>17</v>
       </c>
       <c r="E175" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F175" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G175" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B176" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="C176">
         <v>179</v>
@@ -6290,7 +6415,7 @@
         <v>17</v>
       </c>
       <c r="E176" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="F176" t="s">
         <v>11</v>
@@ -6298,10 +6423,10 @@
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B177" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="C177">
         <v>180</v>
@@ -6318,10 +6443,10 @@
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B178" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="C178">
         <v>181</v>
@@ -6338,10 +6463,10 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B179" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="C179">
         <v>182</v>
@@ -6350,7 +6475,7 @@
         <v>17</v>
       </c>
       <c r="E179" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="F179" t="s">
         <v>11</v>
@@ -6358,10 +6483,10 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B180" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="C180">
         <v>183</v>
@@ -6370,18 +6495,18 @@
         <v>53</v>
       </c>
       <c r="E180" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="F180" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B181" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C181">
         <v>184</v>
@@ -6390,7 +6515,7 @@
         <v>43</v>
       </c>
       <c r="E181" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F181" t="s">
         <v>11</v>
@@ -6398,10 +6523,10 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B182" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="C182">
         <v>185</v>
@@ -6410,18 +6535,18 @@
         <v>37</v>
       </c>
       <c r="E182" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="F182" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B183" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="C183">
         <v>186</v>
@@ -6430,18 +6555,18 @@
         <v>21</v>
       </c>
       <c r="E183" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F183" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B184" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="C184">
         <v>187</v>
@@ -6450,18 +6575,18 @@
         <v>21</v>
       </c>
       <c r="E184" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="F184" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B185" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C185">
         <v>189</v>
@@ -6470,10 +6595,10 @@
         <v>17</v>
       </c>
       <c r="E185" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="F185" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.3">
@@ -6490,18 +6615,18 @@
         <v>53</v>
       </c>
       <c r="E186" t="s">
-        <v>779</v>
+        <v>497</v>
       </c>
       <c r="F186" t="s">
-        <v>11</v>
+        <v>238</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="B187" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="C187">
         <v>191</v>
@@ -6510,7 +6635,7 @@
         <v>9</v>
       </c>
       <c r="E187" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="F187" t="s">
         <v>11</v>
@@ -6518,10 +6643,10 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B188" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="C188">
         <v>192</v>
@@ -6530,18 +6655,18 @@
         <v>43</v>
       </c>
       <c r="E188" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="F188" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="B189" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="C189">
         <v>193</v>
@@ -6550,18 +6675,18 @@
         <v>21</v>
       </c>
       <c r="E189" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F189" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B190" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="C190">
         <v>194</v>
@@ -6570,18 +6695,18 @@
         <v>21</v>
       </c>
       <c r="E190" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F190" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="B191" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="C191">
         <v>195</v>
@@ -6590,18 +6715,18 @@
         <v>21</v>
       </c>
       <c r="E191" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="F191" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B192" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="C192">
         <v>196</v>
@@ -6618,10 +6743,10 @@
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B193" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="C193">
         <v>197</v>
@@ -6630,18 +6755,18 @@
         <v>21</v>
       </c>
       <c r="E193" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="F193" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="B194" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="C194">
         <v>198</v>
@@ -6650,18 +6775,18 @@
         <v>17</v>
       </c>
       <c r="E194" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="F194" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B195" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="C195">
         <v>199</v>
@@ -6678,10 +6803,10 @@
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B196" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="C196">
         <v>200</v>
@@ -6690,18 +6815,18 @@
         <v>43</v>
       </c>
       <c r="E196" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="F196" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="B197" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="C197">
         <v>202</v>
@@ -6710,18 +6835,18 @@
         <v>43</v>
       </c>
       <c r="E197" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="F197" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B198" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="C198">
         <v>203</v>
@@ -6730,18 +6855,18 @@
         <v>53</v>
       </c>
       <c r="E198" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="F198" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="B199" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="C199">
         <v>204</v>
@@ -6750,18 +6875,18 @@
         <v>21</v>
       </c>
       <c r="E199" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="F199" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B200" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="C200">
         <v>205</v>
@@ -6770,18 +6895,18 @@
         <v>53</v>
       </c>
       <c r="E200" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="F200" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="B201" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="C201">
         <v>206</v>
@@ -6790,18 +6915,18 @@
         <v>43</v>
       </c>
       <c r="E201" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="F201" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="B202" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="C202">
         <v>208</v>
@@ -6810,18 +6935,18 @@
         <v>17</v>
       </c>
       <c r="E202" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="F202" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="B203" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="C203">
         <v>209</v>
@@ -6830,18 +6955,18 @@
         <v>53</v>
       </c>
       <c r="E203" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="F203" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="B204" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="C204">
         <v>210</v>
@@ -6850,18 +6975,18 @@
         <v>43</v>
       </c>
       <c r="E204" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="F204" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="B205" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="C205">
         <v>213</v>
@@ -6870,18 +6995,18 @@
         <v>53</v>
       </c>
       <c r="E205" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="F205" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="B206" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="C206">
         <v>214</v>
@@ -6890,18 +7015,18 @@
         <v>21</v>
       </c>
       <c r="E206" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="F206" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B207" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="C207">
         <v>215</v>
@@ -6910,38 +7035,38 @@
         <v>21</v>
       </c>
       <c r="E207" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="F207" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B208" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="C208">
         <v>216</v>
       </c>
       <c r="D208" t="s">
-        <v>21</v>
+        <v>826</v>
       </c>
       <c r="E208" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="F208" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="B209" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="C209">
         <v>217</v>
@@ -6950,18 +7075,18 @@
         <v>17</v>
       </c>
       <c r="E209" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="F209" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="B210" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="C210">
         <v>218</v>
@@ -6970,18 +7095,18 @@
         <v>53</v>
       </c>
       <c r="E210" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="F210" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="B211" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="C211">
         <v>219</v>
@@ -6990,35 +7115,35 @@
         <v>21</v>
       </c>
       <c r="E211" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="F211" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="212" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="B212" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="D212" t="s">
         <v>9</v>
       </c>
       <c r="E212" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="F212" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="B213" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D213" t="s">
         <v>9</v>
@@ -7027,49 +7152,55 @@
         <v>14</v>
       </c>
       <c r="F213" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="B214" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="D214" t="s">
         <v>21</v>
       </c>
       <c r="E214" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="F214" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B215" t="s">
-        <v>577</v>
+        <v>580</v>
+      </c>
+      <c r="C215">
+        <v>231</v>
       </c>
       <c r="D215" t="s">
-        <v>78</v>
+        <v>432</v>
       </c>
       <c r="E215" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="F215" t="s">
-        <v>229</v>
+        <v>238</v>
+      </c>
+      <c r="G215" t="s">
+        <v>582</v>
       </c>
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="B216" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="D216" t="s">
         <v>9</v>
@@ -7078,49 +7209,49 @@
         <v>14</v>
       </c>
       <c r="F216" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="B217" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="D217" t="s">
         <v>9</v>
       </c>
       <c r="E217" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="F217" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="B218" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="D218" t="s">
         <v>21</v>
       </c>
       <c r="E218" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="F218" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="B219" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="D219" t="s">
         <v>21</v>
@@ -7134,30 +7265,33 @@
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="B220" t="s">
-        <v>590</v>
+        <v>594</v>
+      </c>
+      <c r="C220">
+        <v>227</v>
       </c>
       <c r="D220" t="s">
-        <v>777</v>
+        <v>9</v>
       </c>
       <c r="E220" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="F220" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G220" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="B221" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="D221" t="s">
         <v>9</v>
@@ -7166,15 +7300,15 @@
         <v>14</v>
       </c>
       <c r="F221" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="B222" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="D222" t="s">
         <v>21</v>
@@ -7183,32 +7317,32 @@
         <v>14</v>
       </c>
       <c r="F222" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="B223" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="D223" t="s">
         <v>9</v>
       </c>
       <c r="E223" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="F223" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="B224" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="D224" t="s">
         <v>9</v>
@@ -7217,15 +7351,15 @@
         <v>14</v>
       </c>
       <c r="F224" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="B225" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="C225">
         <v>212</v>
@@ -7234,44 +7368,44 @@
         <v>43</v>
       </c>
       <c r="E225" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="F225" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G225" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="B226" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="D226" t="s">
         <v>21</v>
       </c>
       <c r="E226" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="F226" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="B227" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="D227" t="s">
         <v>9</v>
       </c>
       <c r="E227" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="F227" t="s">
         <v>11</v>
@@ -7279,10 +7413,10 @@
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="B228" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="D228" t="s">
         <v>9</v>
@@ -7291,72 +7425,72 @@
         <v>14</v>
       </c>
       <c r="F228" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="B229" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D229" t="s">
         <v>9</v>
       </c>
       <c r="E229" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="F229" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="B230" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="D230" t="s">
         <v>9</v>
       </c>
       <c r="E230" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="F230" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B231" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="D231" t="s">
         <v>9</v>
       </c>
       <c r="E231" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="F231" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="B232" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="D232" t="s">
         <v>9</v>
       </c>
       <c r="E232" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="F232" t="s">
         <v>11</v>
@@ -7364,10 +7498,10 @@
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="B233" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="D233" t="s">
         <v>9</v>
@@ -7381,10 +7515,10 @@
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="B234" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="C234">
         <v>201</v>
@@ -7393,41 +7527,44 @@
         <v>43</v>
       </c>
       <c r="E234" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="F234" t="s">
-        <v>229</v>
+        <v>238</v>
+      </c>
+      <c r="G234" t="s">
+        <v>635</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
-        <v>631</v>
+        <v>636</v>
       </c>
       <c r="B235" t="s">
-        <v>632</v>
+        <v>637</v>
       </c>
       <c r="D235" t="s">
         <v>9</v>
       </c>
       <c r="E235" t="s">
-        <v>633</v>
+        <v>638</v>
       </c>
       <c r="F235" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
-        <v>634</v>
+        <v>639</v>
       </c>
       <c r="B236" t="s">
-        <v>635</v>
+        <v>640</v>
       </c>
       <c r="D236" t="s">
         <v>9</v>
       </c>
       <c r="E236" t="s">
-        <v>636</v>
+        <v>641</v>
       </c>
       <c r="F236" t="s">
         <v>11</v>
@@ -7435,33 +7572,33 @@
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
-        <v>637</v>
+        <v>642</v>
       </c>
       <c r="B237" t="s">
-        <v>638</v>
+        <v>643</v>
       </c>
       <c r="D237" t="s">
         <v>9</v>
       </c>
       <c r="E237" t="s">
-        <v>639</v>
+        <v>644</v>
       </c>
       <c r="F237" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
-        <v>640</v>
+        <v>645</v>
       </c>
       <c r="B238" t="s">
-        <v>641</v>
+        <v>646</v>
       </c>
       <c r="D238" t="s">
         <v>9</v>
       </c>
       <c r="E238" t="s">
-        <v>642</v>
+        <v>647</v>
       </c>
       <c r="F238" t="s">
         <v>11</v>
@@ -7469,16 +7606,16 @@
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
-        <v>643</v>
+        <v>648</v>
       </c>
       <c r="B239" t="s">
-        <v>644</v>
+        <v>649</v>
       </c>
       <c r="D239" t="s">
         <v>9</v>
       </c>
       <c r="E239" t="s">
-        <v>645</v>
+        <v>650</v>
       </c>
       <c r="F239" t="s">
         <v>11</v>
@@ -7486,10 +7623,10 @@
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
-        <v>646</v>
+        <v>651</v>
       </c>
       <c r="B240" t="s">
-        <v>647</v>
+        <v>652</v>
       </c>
       <c r="D240" t="s">
         <v>9</v>
@@ -7498,15 +7635,15 @@
         <v>14</v>
       </c>
       <c r="F240" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
-        <v>648</v>
+        <v>653</v>
       </c>
       <c r="B241" t="s">
-        <v>649</v>
+        <v>654</v>
       </c>
       <c r="D241" t="s">
         <v>9</v>
@@ -7515,15 +7652,15 @@
         <v>14</v>
       </c>
       <c r="F241" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
-        <v>650</v>
+        <v>655</v>
       </c>
       <c r="B242" t="s">
-        <v>651</v>
+        <v>656</v>
       </c>
       <c r="D242" t="s">
         <v>9</v>
@@ -7532,46 +7669,46 @@
         <v>14</v>
       </c>
       <c r="F242" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
-        <v>652</v>
+        <v>657</v>
       </c>
       <c r="B243" t="s">
-        <v>653</v>
+        <v>658</v>
       </c>
       <c r="D243" t="s">
         <v>9</v>
       </c>
       <c r="E243" t="s">
-        <v>654</v>
+        <v>659</v>
       </c>
       <c r="F243" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
-        <v>655</v>
+        <v>660</v>
       </c>
       <c r="B244" t="s">
-        <v>656</v>
+        <v>661</v>
       </c>
       <c r="D244" t="s">
         <v>9</v>
       </c>
       <c r="E244" t="s">
-        <v>657</v>
+        <v>662</v>
       </c>
       <c r="F244" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
-        <v>658</v>
+        <v>663</v>
       </c>
       <c r="B245" t="s">
         <v>290</v>
@@ -7580,103 +7717,109 @@
         <v>9</v>
       </c>
       <c r="E245" t="s">
-        <v>659</v>
+        <v>664</v>
       </c>
       <c r="F245" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
-        <v>660</v>
+        <v>665</v>
       </c>
       <c r="B246" t="s">
-        <v>661</v>
+        <v>666</v>
+      </c>
+      <c r="C246">
+        <v>228</v>
       </c>
       <c r="D246" t="s">
         <v>21</v>
       </c>
       <c r="E246" t="s">
-        <v>662</v>
+        <v>667</v>
       </c>
       <c r="F246" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
-        <v>663</v>
+        <v>668</v>
       </c>
       <c r="B247" t="s">
-        <v>664</v>
+        <v>669</v>
       </c>
       <c r="D247" t="s">
         <v>9</v>
       </c>
       <c r="E247" t="s">
-        <v>665</v>
+        <v>670</v>
       </c>
       <c r="F247" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
-        <v>666</v>
+        <v>671</v>
       </c>
       <c r="B248" t="s">
-        <v>667</v>
+        <v>672</v>
       </c>
       <c r="D248" t="s">
         <v>9</v>
       </c>
       <c r="E248" t="s">
-        <v>668</v>
+        <v>673</v>
       </c>
       <c r="F248" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
-        <v>669</v>
+        <v>674</v>
       </c>
       <c r="B249" t="s">
-        <v>670</v>
+        <v>675</v>
       </c>
       <c r="D249" t="s">
         <v>9</v>
       </c>
       <c r="E249" t="s">
-        <v>671</v>
+        <v>676</v>
       </c>
       <c r="F249" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
-        <v>672</v>
+        <v>677</v>
       </c>
       <c r="B250" t="s">
-        <v>673</v>
+        <v>678</v>
       </c>
       <c r="D250" t="s">
         <v>9</v>
       </c>
       <c r="E250" t="s">
-        <v>674</v>
+        <v>679</v>
       </c>
       <c r="F250" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="G250" t="s">
+        <v>680</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
-        <v>675</v>
+        <v>681</v>
       </c>
       <c r="B251" t="s">
-        <v>676</v>
+        <v>682</v>
       </c>
       <c r="C251">
         <v>207</v>
@@ -7685,35 +7828,35 @@
         <v>53</v>
       </c>
       <c r="E251" t="s">
-        <v>677</v>
+        <v>683</v>
       </c>
       <c r="F251" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
-        <v>678</v>
+        <v>684</v>
       </c>
       <c r="B252" t="s">
-        <v>679</v>
+        <v>685</v>
       </c>
       <c r="D252" t="s">
         <v>17</v>
       </c>
       <c r="E252" t="s">
-        <v>680</v>
+        <v>686</v>
       </c>
       <c r="F252" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="253" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
-        <v>681</v>
+        <v>687</v>
       </c>
       <c r="B253" t="s">
-        <v>682</v>
+        <v>688</v>
       </c>
       <c r="C253">
         <v>211</v>
@@ -7722,205 +7865,208 @@
         <v>17</v>
       </c>
       <c r="E253" t="s">
-        <v>683</v>
+        <v>689</v>
       </c>
       <c r="F253" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
-        <v>684</v>
+        <v>690</v>
       </c>
       <c r="B254" t="s">
-        <v>685</v>
+        <v>691</v>
       </c>
       <c r="D254" t="s">
         <v>9</v>
       </c>
       <c r="E254" t="s">
-        <v>686</v>
+        <v>692</v>
       </c>
       <c r="F254" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="255" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
-        <v>687</v>
+        <v>693</v>
       </c>
       <c r="B255" t="s">
-        <v>688</v>
+        <v>694</v>
       </c>
       <c r="D255" t="s">
         <v>53</v>
       </c>
       <c r="E255" t="s">
-        <v>689</v>
+        <v>695</v>
       </c>
       <c r="F255" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="256" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
-        <v>690</v>
+        <v>696</v>
       </c>
       <c r="B256" t="s">
-        <v>691</v>
+        <v>697</v>
       </c>
       <c r="D256" t="s">
         <v>9</v>
       </c>
       <c r="E256" t="s">
-        <v>692</v>
+        <v>698</v>
       </c>
       <c r="F256" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
-        <v>693</v>
+        <v>699</v>
       </c>
       <c r="B257" t="s">
-        <v>694</v>
+        <v>700</v>
+      </c>
+      <c r="C257">
+        <v>230</v>
       </c>
       <c r="D257" t="s">
         <v>53</v>
       </c>
       <c r="E257" t="s">
-        <v>695</v>
+        <v>701</v>
       </c>
       <c r="F257" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
-        <v>696</v>
+        <v>702</v>
       </c>
       <c r="B258" t="s">
-        <v>697</v>
+        <v>703</v>
       </c>
       <c r="D258" t="s">
         <v>9</v>
       </c>
       <c r="E258" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="F258" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
-        <v>699</v>
+        <v>705</v>
       </c>
       <c r="B259" t="s">
-        <v>700</v>
+        <v>706</v>
       </c>
       <c r="D259" t="s">
         <v>9</v>
       </c>
       <c r="E259" t="s">
-        <v>701</v>
+        <v>707</v>
       </c>
       <c r="F259" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
-        <v>702</v>
+        <v>708</v>
       </c>
       <c r="B260" t="s">
-        <v>703</v>
+        <v>709</v>
       </c>
       <c r="D260" t="s">
         <v>9</v>
       </c>
       <c r="E260" t="s">
-        <v>704</v>
+        <v>710</v>
       </c>
       <c r="F260" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
-        <v>705</v>
+        <v>711</v>
       </c>
       <c r="B261" t="s">
-        <v>706</v>
+        <v>712</v>
       </c>
       <c r="D261" t="s">
         <v>9</v>
       </c>
       <c r="E261" t="s">
-        <v>707</v>
+        <v>713</v>
       </c>
       <c r="F261" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
-        <v>708</v>
+        <v>714</v>
       </c>
       <c r="B262" t="s">
-        <v>709</v>
+        <v>715</v>
       </c>
       <c r="D262" t="s">
         <v>9</v>
       </c>
       <c r="E262" t="s">
-        <v>710</v>
+        <v>716</v>
       </c>
       <c r="F262" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
-        <v>711</v>
+        <v>717</v>
       </c>
       <c r="B263" t="s">
-        <v>712</v>
+        <v>718</v>
       </c>
       <c r="D263" t="s">
         <v>9</v>
       </c>
       <c r="E263" t="s">
-        <v>713</v>
+        <v>719</v>
       </c>
       <c r="F263" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
-        <v>714</v>
+        <v>720</v>
       </c>
       <c r="B264" t="s">
-        <v>715</v>
+        <v>721</v>
       </c>
       <c r="D264" t="s">
         <v>9</v>
       </c>
       <c r="E264" t="s">
-        <v>716</v>
+        <v>722</v>
       </c>
       <c r="F264" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
-        <v>717</v>
+        <v>723</v>
       </c>
       <c r="B265" t="s">
-        <v>718</v>
+        <v>724</v>
       </c>
       <c r="D265" t="s">
         <v>9</v>
@@ -7929,137 +8075,140 @@
         <v>14</v>
       </c>
       <c r="F265" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
-        <v>719</v>
+        <v>725</v>
       </c>
       <c r="B266" t="s">
-        <v>720</v>
+        <v>726</v>
       </c>
       <c r="D266" t="s">
         <v>9</v>
       </c>
       <c r="E266" t="s">
-        <v>721</v>
+        <v>727</v>
       </c>
       <c r="F266" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
-        <v>722</v>
+        <v>728</v>
       </c>
       <c r="B267" t="s">
-        <v>723</v>
+        <v>729</v>
       </c>
       <c r="D267" t="s">
         <v>17</v>
       </c>
       <c r="E267" t="s">
-        <v>724</v>
+        <v>730</v>
       </c>
       <c r="F267" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
-        <v>725</v>
+        <v>731</v>
       </c>
       <c r="B268" t="s">
-        <v>726</v>
+        <v>732</v>
       </c>
       <c r="D268" t="s">
         <v>9</v>
       </c>
       <c r="E268" t="s">
-        <v>727</v>
+        <v>733</v>
       </c>
       <c r="F268" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
-        <v>728</v>
+        <v>734</v>
       </c>
       <c r="B269" t="s">
-        <v>729</v>
+        <v>735</v>
       </c>
       <c r="D269" t="s">
-        <v>777</v>
+        <v>9</v>
       </c>
       <c r="E269" t="s">
-        <v>730</v>
+        <v>736</v>
       </c>
       <c r="F269" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G269" t="s">
-        <v>731</v>
+        <v>737</v>
       </c>
     </row>
     <row r="270" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
-        <v>732</v>
+        <v>738</v>
       </c>
       <c r="B270" t="s">
-        <v>733</v>
+        <v>739</v>
       </c>
       <c r="D270" t="s">
         <v>9</v>
       </c>
       <c r="E270" t="s">
-        <v>734</v>
+        <v>740</v>
       </c>
       <c r="F270" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="271" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
-        <v>735</v>
+        <v>741</v>
       </c>
       <c r="B271" t="s">
-        <v>736</v>
+        <v>742</v>
       </c>
       <c r="D271" t="s">
         <v>9</v>
       </c>
       <c r="E271" t="s">
-        <v>737</v>
+        <v>743</v>
       </c>
       <c r="F271" t="s">
-        <v>229</v>
+        <v>238</v>
+      </c>
+      <c r="G271" t="s">
+        <v>744</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
-        <v>738</v>
+        <v>745</v>
       </c>
       <c r="B272" t="s">
-        <v>739</v>
+        <v>746</v>
       </c>
       <c r="D272" t="s">
         <v>9</v>
       </c>
       <c r="E272" t="s">
-        <v>740</v>
+        <v>747</v>
       </c>
       <c r="F272" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
-        <v>741</v>
+        <v>748</v>
       </c>
       <c r="B273" t="s">
-        <v>742</v>
+        <v>749</v>
       </c>
       <c r="C273">
         <v>220</v>
@@ -8076,16 +8225,16 @@
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
-        <v>743</v>
+        <v>750</v>
       </c>
       <c r="B274" t="s">
-        <v>744</v>
+        <v>751</v>
       </c>
       <c r="D274" t="s">
         <v>9</v>
       </c>
       <c r="E274" t="s">
-        <v>745</v>
+        <v>752</v>
       </c>
       <c r="F274" t="s">
         <v>11</v>
@@ -8093,27 +8242,27 @@
     </row>
     <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
-        <v>746</v>
+        <v>753</v>
       </c>
       <c r="B275" t="s">
-        <v>747</v>
+        <v>754</v>
       </c>
       <c r="D275" t="s">
         <v>9</v>
       </c>
       <c r="E275" t="s">
-        <v>748</v>
+        <v>755</v>
       </c>
       <c r="F275" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
-        <v>749</v>
+        <v>756</v>
       </c>
       <c r="B276" t="s">
-        <v>750</v>
+        <v>757</v>
       </c>
       <c r="C276">
         <v>196</v>
@@ -8122,75 +8271,75 @@
         <v>17</v>
       </c>
       <c r="E276" t="s">
-        <v>751</v>
+        <v>758</v>
       </c>
       <c r="F276" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G276" t="s">
-        <v>752</v>
+        <v>759</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
-        <v>753</v>
+        <v>760</v>
       </c>
       <c r="B277" t="s">
-        <v>754</v>
+        <v>761</v>
       </c>
       <c r="D277" t="s">
         <v>9</v>
       </c>
       <c r="E277" t="s">
-        <v>755</v>
+        <v>762</v>
       </c>
       <c r="F277" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
-        <v>756</v>
+        <v>763</v>
       </c>
       <c r="B278" t="s">
-        <v>757</v>
+        <v>764</v>
       </c>
       <c r="D278" t="s">
         <v>9</v>
       </c>
       <c r="E278" t="s">
-        <v>758</v>
+        <v>765</v>
       </c>
       <c r="F278" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
-        <v>759</v>
+        <v>766</v>
       </c>
       <c r="B279" t="s">
-        <v>760</v>
+        <v>767</v>
       </c>
       <c r="D279" t="s">
         <v>21</v>
       </c>
       <c r="E279" t="s">
-        <v>761</v>
+        <v>768</v>
       </c>
       <c r="F279" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G279" t="s">
-        <v>762</v>
+        <v>824</v>
       </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="B280" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="D280" t="s">
         <v>9</v>
@@ -8199,97 +8348,369 @@
         <v>14</v>
       </c>
       <c r="F280" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
-        <v>765</v>
+        <v>771</v>
       </c>
       <c r="B281" t="s">
-        <v>766</v>
+        <v>772</v>
       </c>
       <c r="D281" t="s">
         <v>9</v>
       </c>
       <c r="E281" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="F281" t="s">
-        <v>229</v>
+        <v>11</v>
       </c>
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
-        <v>768</v>
+        <v>774</v>
       </c>
       <c r="B282" t="s">
-        <v>769</v>
+        <v>775</v>
       </c>
       <c r="D282" t="s">
         <v>17</v>
       </c>
       <c r="E282" t="s">
-        <v>770</v>
+        <v>776</v>
       </c>
       <c r="F282" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
-        <v>771</v>
+        <v>777</v>
       </c>
       <c r="B283" t="s">
-        <v>772</v>
+        <v>778</v>
       </c>
       <c r="D283" t="s">
         <v>9</v>
       </c>
       <c r="E283" t="s">
-        <v>773</v>
+        <v>779</v>
       </c>
       <c r="F283" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
-        <v>774</v>
+        <v>780</v>
       </c>
       <c r="B284" t="s">
-        <v>775</v>
+        <v>781</v>
       </c>
       <c r="D284" t="s">
         <v>9</v>
       </c>
       <c r="E284" t="s">
-        <v>776</v>
+        <v>782</v>
       </c>
       <c r="F284" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
-        <v>782</v>
+        <v>783</v>
       </c>
       <c r="B285" t="s">
-        <v>783</v>
+        <v>784</v>
       </c>
       <c r="D285" t="s">
-        <v>781</v>
+        <v>17</v>
       </c>
       <c r="E285" t="s">
         <v>14</v>
       </c>
       <c r="F285" t="s">
         <v>11</v>
+      </c>
+    </row>
+    <row r="286" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A286" t="s">
+        <v>785</v>
+      </c>
+      <c r="B286" t="s">
+        <v>786</v>
+      </c>
+      <c r="D286" t="s">
+        <v>9</v>
+      </c>
+      <c r="E286" t="s">
+        <v>787</v>
+      </c>
+      <c r="F286" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="287" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A287" t="s">
+        <v>788</v>
+      </c>
+      <c r="B287" t="s">
+        <v>789</v>
+      </c>
+      <c r="D287" t="s">
+        <v>9</v>
+      </c>
+      <c r="E287" t="s">
+        <v>790</v>
+      </c>
+      <c r="F287" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="288" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A288" t="s">
+        <v>791</v>
+      </c>
+      <c r="B288" t="s">
+        <v>167</v>
+      </c>
+      <c r="D288" t="s">
+        <v>17</v>
+      </c>
+      <c r="E288" t="s">
+        <v>792</v>
+      </c>
+      <c r="F288" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="289" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A289" t="s">
+        <v>793</v>
+      </c>
+      <c r="B289" t="s">
+        <v>794</v>
+      </c>
+      <c r="D289" t="s">
+        <v>9</v>
+      </c>
+      <c r="E289" t="s">
+        <v>795</v>
+      </c>
+      <c r="F289" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="290" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A290" t="s">
+        <v>796</v>
+      </c>
+      <c r="B290" t="s">
+        <v>797</v>
+      </c>
+      <c r="D290" t="s">
+        <v>9</v>
+      </c>
+      <c r="E290" t="s">
+        <v>798</v>
+      </c>
+      <c r="F290" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="291" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A291" t="s">
+        <v>799</v>
+      </c>
+      <c r="B291" t="s">
+        <v>800</v>
+      </c>
+      <c r="D291" t="s">
+        <v>9</v>
+      </c>
+      <c r="E291" t="s">
+        <v>801</v>
+      </c>
+      <c r="F291" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="292" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A292" t="s">
+        <v>802</v>
+      </c>
+      <c r="B292" t="s">
+        <v>803</v>
+      </c>
+      <c r="D292" t="s">
+        <v>9</v>
+      </c>
+      <c r="E292" t="s">
+        <v>804</v>
+      </c>
+      <c r="F292" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="293" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A293" t="s">
+        <v>805</v>
+      </c>
+      <c r="B293" t="s">
+        <v>806</v>
+      </c>
+      <c r="D293" t="s">
+        <v>9</v>
+      </c>
+      <c r="E293" t="s">
+        <v>807</v>
+      </c>
+      <c r="F293" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="294" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A294" t="s">
+        <v>808</v>
+      </c>
+      <c r="B294" t="s">
+        <v>809</v>
+      </c>
+      <c r="D294" t="s">
+        <v>17</v>
+      </c>
+      <c r="E294" t="s">
+        <v>14</v>
+      </c>
+      <c r="F294" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="295" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A295" t="s">
+        <v>825</v>
+      </c>
+      <c r="B295" t="s">
+        <v>810</v>
+      </c>
+      <c r="D295" t="s">
+        <v>17</v>
+      </c>
+      <c r="E295" t="s">
+        <v>14</v>
+      </c>
+      <c r="F295" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="296" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A296" t="s">
+        <v>811</v>
+      </c>
+      <c r="B296" t="s">
+        <v>812</v>
+      </c>
+      <c r="D296" t="s">
+        <v>17</v>
+      </c>
+      <c r="E296" t="s">
+        <v>14</v>
+      </c>
+      <c r="F296" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="297" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A297" t="s">
+        <v>813</v>
+      </c>
+      <c r="B297" t="s">
+        <v>814</v>
+      </c>
+      <c r="D297" t="s">
+        <v>17</v>
+      </c>
+      <c r="E297" t="s">
+        <v>14</v>
+      </c>
+      <c r="F297" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="298" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A298" t="s">
+        <v>815</v>
+      </c>
+      <c r="B298" t="s">
+        <v>816</v>
+      </c>
+      <c r="D298" t="s">
+        <v>17</v>
+      </c>
+      <c r="E298" t="s">
+        <v>14</v>
+      </c>
+      <c r="F298" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="299" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A299" t="s">
+        <v>817</v>
+      </c>
+      <c r="B299" t="s">
+        <v>818</v>
+      </c>
+      <c r="D299" t="s">
+        <v>37</v>
+      </c>
+      <c r="E299" t="s">
+        <v>819</v>
+      </c>
+      <c r="F299" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="300" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A300" t="s">
+        <v>820</v>
+      </c>
+      <c r="B300" t="s">
+        <v>821</v>
+      </c>
+      <c r="D300" t="s">
+        <v>37</v>
+      </c>
+      <c r="E300" t="s">
+        <v>14</v>
+      </c>
+      <c r="F300" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="301" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A301" t="s">
+        <v>822</v>
+      </c>
+      <c r="B301" t="s">
+        <v>823</v>
+      </c>
+      <c r="D301" t="s">
+        <v>37</v>
+      </c>
+      <c r="E301" t="s">
+        <v>14</v>
+      </c>
+      <c r="F301" t="s">
+        <v>238</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Deploying to gh-pages from @ X-LANCE/x-lance.github.io@753f1e6cc60d30bf1c5a86d8cb00c35292e2a2c7 🚀
</commit_message>
<xml_diff>
--- a/process_avatar/final.xlsx
+++ b/process_avatar/final.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SJTU\X-LANCE\宣传委员\xlance.github.io\process_avatar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1A2496-B6E7-4D8D-A06C-54BFC45B3733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C091AF9-5474-41FA-AC8F-045208F6F500}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38510" yWindow="-16840" windowWidth="38620" windowHeight="21820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1339,9 +1339,6 @@
     <t>Hanqi Li</t>
   </si>
   <si>
-    <t>/assets/img/members/student/李翰奇.jpg</t>
-  </si>
-  <si>
     <t>孙良泰</t>
   </si>
   <si>
@@ -2503,6 +2500,10 @@
   </si>
   <si>
     <t>UM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>/assets/img/members/student/李翰奇_2.jpg</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -6206,7 +6207,7 @@
         <v>43</v>
       </c>
       <c r="E166" t="s">
-        <v>439</v>
+        <v>826</v>
       </c>
       <c r="F166" t="s">
         <v>238</v>
@@ -6214,10 +6215,10 @@
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
+        <v>439</v>
+      </c>
+      <c r="B167" t="s">
         <v>440</v>
-      </c>
-      <c r="B167" t="s">
-        <v>441</v>
       </c>
       <c r="C167">
         <v>170</v>
@@ -6226,7 +6227,7 @@
         <v>21</v>
       </c>
       <c r="E167" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
       <c r="F167" t="s">
         <v>11</v>
@@ -6234,10 +6235,10 @@
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
+        <v>442</v>
+      </c>
+      <c r="B168" t="s">
         <v>443</v>
-      </c>
-      <c r="B168" t="s">
-        <v>444</v>
       </c>
       <c r="C168">
         <v>171</v>
@@ -6246,21 +6247,21 @@
         <v>53</v>
       </c>
       <c r="E168" t="s">
+        <v>444</v>
+      </c>
+      <c r="F168" t="s">
+        <v>238</v>
+      </c>
+      <c r="G168" t="s">
         <v>445</v>
-      </c>
-      <c r="F168" t="s">
-        <v>238</v>
-      </c>
-      <c r="G168" t="s">
-        <v>446</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
+        <v>446</v>
+      </c>
+      <c r="B169" t="s">
         <v>447</v>
-      </c>
-      <c r="B169" t="s">
-        <v>448</v>
       </c>
       <c r="C169">
         <v>172</v>
@@ -6269,7 +6270,7 @@
         <v>17</v>
       </c>
       <c r="E169" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="F169" t="s">
         <v>11</v>
@@ -6277,10 +6278,10 @@
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
+        <v>449</v>
+      </c>
+      <c r="B170" t="s">
         <v>450</v>
-      </c>
-      <c r="B170" t="s">
-        <v>451</v>
       </c>
       <c r="C170">
         <v>173</v>
@@ -6289,7 +6290,7 @@
         <v>17</v>
       </c>
       <c r="E170" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="F170" t="s">
         <v>11</v>
@@ -6297,10 +6298,10 @@
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
+        <v>452</v>
+      </c>
+      <c r="B171" t="s">
         <v>453</v>
-      </c>
-      <c r="B171" t="s">
-        <v>454</v>
       </c>
       <c r="C171">
         <v>174</v>
@@ -6317,10 +6318,10 @@
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
+        <v>454</v>
+      </c>
+      <c r="B172" t="s">
         <v>455</v>
-      </c>
-      <c r="B172" t="s">
-        <v>456</v>
       </c>
       <c r="C172">
         <v>175</v>
@@ -6329,7 +6330,7 @@
         <v>17</v>
       </c>
       <c r="E172" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="F172" t="s">
         <v>11</v>
@@ -6337,10 +6338,10 @@
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
+        <v>457</v>
+      </c>
+      <c r="B173" t="s">
         <v>458</v>
-      </c>
-      <c r="B173" t="s">
-        <v>459</v>
       </c>
       <c r="C173">
         <v>176</v>
@@ -6349,7 +6350,7 @@
         <v>17</v>
       </c>
       <c r="E173" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F173" t="s">
         <v>11</v>
@@ -6357,10 +6358,10 @@
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
+        <v>460</v>
+      </c>
+      <c r="B174" t="s">
         <v>461</v>
-      </c>
-      <c r="B174" t="s">
-        <v>462</v>
       </c>
       <c r="C174">
         <v>177</v>
@@ -6369,21 +6370,21 @@
         <v>43</v>
       </c>
       <c r="E174" t="s">
+        <v>462</v>
+      </c>
+      <c r="F174" t="s">
+        <v>238</v>
+      </c>
+      <c r="G174" t="s">
         <v>463</v>
-      </c>
-      <c r="F174" t="s">
-        <v>238</v>
-      </c>
-      <c r="G174" t="s">
-        <v>464</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
+        <v>464</v>
+      </c>
+      <c r="B175" t="s">
         <v>465</v>
-      </c>
-      <c r="B175" t="s">
-        <v>466</v>
       </c>
       <c r="C175">
         <v>178</v>
@@ -6392,21 +6393,21 @@
         <v>17</v>
       </c>
       <c r="E175" t="s">
+        <v>466</v>
+      </c>
+      <c r="F175" t="s">
+        <v>238</v>
+      </c>
+      <c r="G175" t="s">
         <v>467</v>
-      </c>
-      <c r="F175" t="s">
-        <v>238</v>
-      </c>
-      <c r="G175" t="s">
-        <v>468</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
+        <v>468</v>
+      </c>
+      <c r="B176" t="s">
         <v>469</v>
-      </c>
-      <c r="B176" t="s">
-        <v>470</v>
       </c>
       <c r="C176">
         <v>179</v>
@@ -6415,7 +6416,7 @@
         <v>17</v>
       </c>
       <c r="E176" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F176" t="s">
         <v>11</v>
@@ -6423,10 +6424,10 @@
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
+        <v>471</v>
+      </c>
+      <c r="B177" t="s">
         <v>472</v>
-      </c>
-      <c r="B177" t="s">
-        <v>473</v>
       </c>
       <c r="C177">
         <v>180</v>
@@ -6443,10 +6444,10 @@
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
+        <v>473</v>
+      </c>
+      <c r="B178" t="s">
         <v>474</v>
-      </c>
-      <c r="B178" t="s">
-        <v>475</v>
       </c>
       <c r="C178">
         <v>181</v>
@@ -6463,10 +6464,10 @@
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
+        <v>475</v>
+      </c>
+      <c r="B179" t="s">
         <v>476</v>
-      </c>
-      <c r="B179" t="s">
-        <v>477</v>
       </c>
       <c r="C179">
         <v>182</v>
@@ -6475,7 +6476,7 @@
         <v>17</v>
       </c>
       <c r="E179" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F179" t="s">
         <v>11</v>
@@ -6483,10 +6484,10 @@
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
+        <v>478</v>
+      </c>
+      <c r="B180" t="s">
         <v>479</v>
-      </c>
-      <c r="B180" t="s">
-        <v>480</v>
       </c>
       <c r="C180">
         <v>183</v>
@@ -6495,7 +6496,7 @@
         <v>53</v>
       </c>
       <c r="E180" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="F180" t="s">
         <v>238</v>
@@ -6503,10 +6504,10 @@
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
+        <v>481</v>
+      </c>
+      <c r="B181" t="s">
         <v>482</v>
-      </c>
-      <c r="B181" t="s">
-        <v>483</v>
       </c>
       <c r="C181">
         <v>184</v>
@@ -6515,7 +6516,7 @@
         <v>43</v>
       </c>
       <c r="E181" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="F181" t="s">
         <v>11</v>
@@ -6523,10 +6524,10 @@
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
+        <v>484</v>
+      </c>
+      <c r="B182" t="s">
         <v>485</v>
-      </c>
-      <c r="B182" t="s">
-        <v>486</v>
       </c>
       <c r="C182">
         <v>185</v>
@@ -6535,7 +6536,7 @@
         <v>37</v>
       </c>
       <c r="E182" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="F182" t="s">
         <v>11</v>
@@ -6543,10 +6544,10 @@
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
+        <v>487</v>
+      </c>
+      <c r="B183" t="s">
         <v>488</v>
-      </c>
-      <c r="B183" t="s">
-        <v>489</v>
       </c>
       <c r="C183">
         <v>186</v>
@@ -6555,7 +6556,7 @@
         <v>21</v>
       </c>
       <c r="E183" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="F183" t="s">
         <v>238</v>
@@ -6563,10 +6564,10 @@
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
+        <v>490</v>
+      </c>
+      <c r="B184" t="s">
         <v>491</v>
-      </c>
-      <c r="B184" t="s">
-        <v>492</v>
       </c>
       <c r="C184">
         <v>187</v>
@@ -6575,7 +6576,7 @@
         <v>21</v>
       </c>
       <c r="E184" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="F184" t="s">
         <v>238</v>
@@ -6583,10 +6584,10 @@
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
+        <v>493</v>
+      </c>
+      <c r="B185" t="s">
         <v>494</v>
-      </c>
-      <c r="B185" t="s">
-        <v>495</v>
       </c>
       <c r="C185">
         <v>189</v>
@@ -6595,7 +6596,7 @@
         <v>17</v>
       </c>
       <c r="E185" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="F185" t="s">
         <v>238</v>
@@ -6615,7 +6616,7 @@
         <v>53</v>
       </c>
       <c r="E186" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="F186" t="s">
         <v>238</v>
@@ -6623,10 +6624,10 @@
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
+        <v>497</v>
+      </c>
+      <c r="B187" t="s">
         <v>498</v>
-      </c>
-      <c r="B187" t="s">
-        <v>499</v>
       </c>
       <c r="C187">
         <v>191</v>
@@ -6635,7 +6636,7 @@
         <v>9</v>
       </c>
       <c r="E187" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="F187" t="s">
         <v>11</v>
@@ -6643,10 +6644,10 @@
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
+        <v>500</v>
+      </c>
+      <c r="B188" t="s">
         <v>501</v>
-      </c>
-      <c r="B188" t="s">
-        <v>502</v>
       </c>
       <c r="C188">
         <v>192</v>
@@ -6655,7 +6656,7 @@
         <v>43</v>
       </c>
       <c r="E188" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="F188" t="s">
         <v>238</v>
@@ -6663,10 +6664,10 @@
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
+        <v>503</v>
+      </c>
+      <c r="B189" t="s">
         <v>504</v>
-      </c>
-      <c r="B189" t="s">
-        <v>505</v>
       </c>
       <c r="C189">
         <v>193</v>
@@ -6675,7 +6676,7 @@
         <v>21</v>
       </c>
       <c r="E189" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="F189" t="s">
         <v>238</v>
@@ -6683,10 +6684,10 @@
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
+        <v>506</v>
+      </c>
+      <c r="B190" t="s">
         <v>507</v>
-      </c>
-      <c r="B190" t="s">
-        <v>508</v>
       </c>
       <c r="C190">
         <v>194</v>
@@ -6695,7 +6696,7 @@
         <v>21</v>
       </c>
       <c r="E190" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="F190" t="s">
         <v>238</v>
@@ -6703,10 +6704,10 @@
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
+        <v>509</v>
+      </c>
+      <c r="B191" t="s">
         <v>510</v>
-      </c>
-      <c r="B191" t="s">
-        <v>511</v>
       </c>
       <c r="C191">
         <v>195</v>
@@ -6715,7 +6716,7 @@
         <v>21</v>
       </c>
       <c r="E191" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="F191" t="s">
         <v>238</v>
@@ -6723,10 +6724,10 @@
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
+        <v>512</v>
+      </c>
+      <c r="B192" t="s">
         <v>513</v>
-      </c>
-      <c r="B192" t="s">
-        <v>514</v>
       </c>
       <c r="C192">
         <v>196</v>
@@ -6743,10 +6744,10 @@
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
+        <v>514</v>
+      </c>
+      <c r="B193" t="s">
         <v>515</v>
-      </c>
-      <c r="B193" t="s">
-        <v>516</v>
       </c>
       <c r="C193">
         <v>197</v>
@@ -6755,7 +6756,7 @@
         <v>21</v>
       </c>
       <c r="E193" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F193" t="s">
         <v>238</v>
@@ -6763,10 +6764,10 @@
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
+        <v>517</v>
+      </c>
+      <c r="B194" t="s">
         <v>518</v>
-      </c>
-      <c r="B194" t="s">
-        <v>519</v>
       </c>
       <c r="C194">
         <v>198</v>
@@ -6775,7 +6776,7 @@
         <v>17</v>
       </c>
       <c r="E194" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="F194" t="s">
         <v>238</v>
@@ -6783,10 +6784,10 @@
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
+        <v>520</v>
+      </c>
+      <c r="B195" t="s">
         <v>521</v>
-      </c>
-      <c r="B195" t="s">
-        <v>522</v>
       </c>
       <c r="C195">
         <v>199</v>
@@ -6803,10 +6804,10 @@
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
+        <v>522</v>
+      </c>
+      <c r="B196" t="s">
         <v>523</v>
-      </c>
-      <c r="B196" t="s">
-        <v>524</v>
       </c>
       <c r="C196">
         <v>200</v>
@@ -6815,7 +6816,7 @@
         <v>43</v>
       </c>
       <c r="E196" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="F196" t="s">
         <v>238</v>
@@ -6823,10 +6824,10 @@
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
+        <v>525</v>
+      </c>
+      <c r="B197" t="s">
         <v>526</v>
-      </c>
-      <c r="B197" t="s">
-        <v>527</v>
       </c>
       <c r="C197">
         <v>202</v>
@@ -6835,7 +6836,7 @@
         <v>43</v>
       </c>
       <c r="E197" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="F197" t="s">
         <v>238</v>
@@ -6843,10 +6844,10 @@
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
+        <v>528</v>
+      </c>
+      <c r="B198" t="s">
         <v>529</v>
-      </c>
-      <c r="B198" t="s">
-        <v>530</v>
       </c>
       <c r="C198">
         <v>203</v>
@@ -6855,7 +6856,7 @@
         <v>53</v>
       </c>
       <c r="E198" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="F198" t="s">
         <v>238</v>
@@ -6863,10 +6864,10 @@
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
+        <v>531</v>
+      </c>
+      <c r="B199" t="s">
         <v>532</v>
-      </c>
-      <c r="B199" t="s">
-        <v>533</v>
       </c>
       <c r="C199">
         <v>204</v>
@@ -6875,7 +6876,7 @@
         <v>21</v>
       </c>
       <c r="E199" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="F199" t="s">
         <v>238</v>
@@ -6883,10 +6884,10 @@
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
+        <v>534</v>
+      </c>
+      <c r="B200" t="s">
         <v>535</v>
-      </c>
-      <c r="B200" t="s">
-        <v>536</v>
       </c>
       <c r="C200">
         <v>205</v>
@@ -6895,7 +6896,7 @@
         <v>53</v>
       </c>
       <c r="E200" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F200" t="s">
         <v>238</v>
@@ -6903,10 +6904,10 @@
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
+        <v>537</v>
+      </c>
+      <c r="B201" t="s">
         <v>538</v>
-      </c>
-      <c r="B201" t="s">
-        <v>539</v>
       </c>
       <c r="C201">
         <v>206</v>
@@ -6915,7 +6916,7 @@
         <v>43</v>
       </c>
       <c r="E201" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="F201" t="s">
         <v>238</v>
@@ -6923,10 +6924,10 @@
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
+        <v>540</v>
+      </c>
+      <c r="B202" t="s">
         <v>541</v>
-      </c>
-      <c r="B202" t="s">
-        <v>542</v>
       </c>
       <c r="C202">
         <v>208</v>
@@ -6935,7 +6936,7 @@
         <v>17</v>
       </c>
       <c r="E202" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="F202" t="s">
         <v>238</v>
@@ -6943,10 +6944,10 @@
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
+        <v>543</v>
+      </c>
+      <c r="B203" t="s">
         <v>544</v>
-      </c>
-      <c r="B203" t="s">
-        <v>545</v>
       </c>
       <c r="C203">
         <v>209</v>
@@ -6955,7 +6956,7 @@
         <v>53</v>
       </c>
       <c r="E203" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F203" t="s">
         <v>238</v>
@@ -6963,10 +6964,10 @@
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
+        <v>546</v>
+      </c>
+      <c r="B204" t="s">
         <v>547</v>
-      </c>
-      <c r="B204" t="s">
-        <v>548</v>
       </c>
       <c r="C204">
         <v>210</v>
@@ -6975,7 +6976,7 @@
         <v>43</v>
       </c>
       <c r="E204" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F204" t="s">
         <v>238</v>
@@ -6983,10 +6984,10 @@
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
+        <v>549</v>
+      </c>
+      <c r="B205" t="s">
         <v>550</v>
-      </c>
-      <c r="B205" t="s">
-        <v>551</v>
       </c>
       <c r="C205">
         <v>213</v>
@@ -6995,7 +6996,7 @@
         <v>53</v>
       </c>
       <c r="E205" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F205" t="s">
         <v>238</v>
@@ -7003,10 +7004,10 @@
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
+        <v>552</v>
+      </c>
+      <c r="B206" t="s">
         <v>553</v>
-      </c>
-      <c r="B206" t="s">
-        <v>554</v>
       </c>
       <c r="C206">
         <v>214</v>
@@ -7015,7 +7016,7 @@
         <v>21</v>
       </c>
       <c r="E206" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F206" t="s">
         <v>238</v>
@@ -7023,10 +7024,10 @@
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
+        <v>555</v>
+      </c>
+      <c r="B207" t="s">
         <v>556</v>
-      </c>
-      <c r="B207" t="s">
-        <v>557</v>
       </c>
       <c r="C207">
         <v>215</v>
@@ -7035,7 +7036,7 @@
         <v>21</v>
       </c>
       <c r="E207" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F207" t="s">
         <v>238</v>
@@ -7043,19 +7044,19 @@
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
+        <v>558</v>
+      </c>
+      <c r="B208" t="s">
         <v>559</v>
-      </c>
-      <c r="B208" t="s">
-        <v>560</v>
       </c>
       <c r="C208">
         <v>216</v>
       </c>
       <c r="D208" t="s">
-        <v>826</v>
+        <v>825</v>
       </c>
       <c r="E208" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F208" t="s">
         <v>238</v>
@@ -7063,10 +7064,10 @@
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
+        <v>561</v>
+      </c>
+      <c r="B209" t="s">
         <v>562</v>
-      </c>
-      <c r="B209" t="s">
-        <v>563</v>
       </c>
       <c r="C209">
         <v>217</v>
@@ -7075,7 +7076,7 @@
         <v>17</v>
       </c>
       <c r="E209" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F209" t="s">
         <v>238</v>
@@ -7083,10 +7084,10 @@
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
+        <v>564</v>
+      </c>
+      <c r="B210" t="s">
         <v>565</v>
-      </c>
-      <c r="B210" t="s">
-        <v>566</v>
       </c>
       <c r="C210">
         <v>218</v>
@@ -7095,7 +7096,7 @@
         <v>53</v>
       </c>
       <c r="E210" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="F210" t="s">
         <v>238</v>
@@ -7103,10 +7104,10 @@
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
+        <v>567</v>
+      </c>
+      <c r="B211" t="s">
         <v>568</v>
-      </c>
-      <c r="B211" t="s">
-        <v>569</v>
       </c>
       <c r="C211">
         <v>219</v>
@@ -7115,7 +7116,7 @@
         <v>21</v>
       </c>
       <c r="E211" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="F211" t="s">
         <v>238</v>
@@ -7123,16 +7124,16 @@
     </row>
     <row r="212" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
+        <v>570</v>
+      </c>
+      <c r="B212" t="s">
         <v>571</v>
       </c>
-      <c r="B212" t="s">
+      <c r="D212" t="s">
+        <v>9</v>
+      </c>
+      <c r="E212" t="s">
         <v>572</v>
-      </c>
-      <c r="D212" t="s">
-        <v>9</v>
-      </c>
-      <c r="E212" t="s">
-        <v>573</v>
       </c>
       <c r="F212" t="s">
         <v>238</v>
@@ -7140,10 +7141,10 @@
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
+        <v>573</v>
+      </c>
+      <c r="B213" t="s">
         <v>574</v>
-      </c>
-      <c r="B213" t="s">
-        <v>575</v>
       </c>
       <c r="D213" t="s">
         <v>9</v>
@@ -7157,16 +7158,16 @@
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
+        <v>575</v>
+      </c>
+      <c r="B214" t="s">
         <v>576</v>
-      </c>
-      <c r="B214" t="s">
-        <v>577</v>
       </c>
       <c r="D214" t="s">
         <v>21</v>
       </c>
       <c r="E214" t="s">
-        <v>578</v>
+        <v>577</v>
       </c>
       <c r="F214" t="s">
         <v>238</v>
@@ -7174,10 +7175,10 @@
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
+        <v>578</v>
+      </c>
+      <c r="B215" t="s">
         <v>579</v>
-      </c>
-      <c r="B215" t="s">
-        <v>580</v>
       </c>
       <c r="C215">
         <v>231</v>
@@ -7186,21 +7187,21 @@
         <v>432</v>
       </c>
       <c r="E215" t="s">
+        <v>580</v>
+      </c>
+      <c r="F215" t="s">
+        <v>238</v>
+      </c>
+      <c r="G215" t="s">
         <v>581</v>
-      </c>
-      <c r="F215" t="s">
-        <v>238</v>
-      </c>
-      <c r="G215" t="s">
-        <v>582</v>
       </c>
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
+        <v>582</v>
+      </c>
+      <c r="B216" t="s">
         <v>583</v>
-      </c>
-      <c r="B216" t="s">
-        <v>584</v>
       </c>
       <c r="D216" t="s">
         <v>9</v>
@@ -7214,16 +7215,16 @@
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
+        <v>584</v>
+      </c>
+      <c r="B217" t="s">
         <v>585</v>
       </c>
-      <c r="B217" t="s">
+      <c r="D217" t="s">
+        <v>9</v>
+      </c>
+      <c r="E217" t="s">
         <v>586</v>
-      </c>
-      <c r="D217" t="s">
-        <v>9</v>
-      </c>
-      <c r="E217" t="s">
-        <v>587</v>
       </c>
       <c r="F217" t="s">
         <v>238</v>
@@ -7231,16 +7232,16 @@
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
+        <v>587</v>
+      </c>
+      <c r="B218" t="s">
         <v>588</v>
-      </c>
-      <c r="B218" t="s">
-        <v>589</v>
       </c>
       <c r="D218" t="s">
         <v>21</v>
       </c>
       <c r="E218" t="s">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="F218" t="s">
         <v>238</v>
@@ -7248,10 +7249,10 @@
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
+        <v>590</v>
+      </c>
+      <c r="B219" t="s">
         <v>591</v>
-      </c>
-      <c r="B219" t="s">
-        <v>592</v>
       </c>
       <c r="D219" t="s">
         <v>21</v>
@@ -7265,10 +7266,10 @@
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
+        <v>592</v>
+      </c>
+      <c r="B220" t="s">
         <v>593</v>
-      </c>
-      <c r="B220" t="s">
-        <v>594</v>
       </c>
       <c r="C220">
         <v>227</v>
@@ -7277,21 +7278,21 @@
         <v>9</v>
       </c>
       <c r="E220" t="s">
+        <v>594</v>
+      </c>
+      <c r="F220" t="s">
+        <v>238</v>
+      </c>
+      <c r="G220" t="s">
         <v>595</v>
-      </c>
-      <c r="F220" t="s">
-        <v>238</v>
-      </c>
-      <c r="G220" t="s">
-        <v>596</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
+        <v>596</v>
+      </c>
+      <c r="B221" t="s">
         <v>597</v>
-      </c>
-      <c r="B221" t="s">
-        <v>598</v>
       </c>
       <c r="D221" t="s">
         <v>9</v>
@@ -7305,10 +7306,10 @@
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
+        <v>598</v>
+      </c>
+      <c r="B222" t="s">
         <v>599</v>
-      </c>
-      <c r="B222" t="s">
-        <v>600</v>
       </c>
       <c r="D222" t="s">
         <v>21</v>
@@ -7322,16 +7323,16 @@
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
+        <v>600</v>
+      </c>
+      <c r="B223" t="s">
         <v>601</v>
       </c>
-      <c r="B223" t="s">
+      <c r="D223" t="s">
+        <v>9</v>
+      </c>
+      <c r="E223" t="s">
         <v>602</v>
-      </c>
-      <c r="D223" t="s">
-        <v>9</v>
-      </c>
-      <c r="E223" t="s">
-        <v>603</v>
       </c>
       <c r="F223" t="s">
         <v>238</v>
@@ -7339,10 +7340,10 @@
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
+        <v>603</v>
+      </c>
+      <c r="B224" t="s">
         <v>604</v>
-      </c>
-      <c r="B224" t="s">
-        <v>605</v>
       </c>
       <c r="D224" t="s">
         <v>9</v>
@@ -7356,10 +7357,10 @@
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
+        <v>605</v>
+      </c>
+      <c r="B225" t="s">
         <v>606</v>
-      </c>
-      <c r="B225" t="s">
-        <v>607</v>
       </c>
       <c r="C225">
         <v>212</v>
@@ -7368,27 +7369,27 @@
         <v>43</v>
       </c>
       <c r="E225" t="s">
+        <v>607</v>
+      </c>
+      <c r="F225" t="s">
+        <v>238</v>
+      </c>
+      <c r="G225" t="s">
         <v>608</v>
-      </c>
-      <c r="F225" t="s">
-        <v>238</v>
-      </c>
-      <c r="G225" t="s">
-        <v>609</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
+        <v>609</v>
+      </c>
+      <c r="B226" t="s">
         <v>610</v>
-      </c>
-      <c r="B226" t="s">
-        <v>611</v>
       </c>
       <c r="D226" t="s">
         <v>21</v>
       </c>
       <c r="E226" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="F226" t="s">
         <v>11</v>
@@ -7396,16 +7397,16 @@
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
+        <v>612</v>
+      </c>
+      <c r="B227" t="s">
         <v>613</v>
       </c>
-      <c r="B227" t="s">
+      <c r="D227" t="s">
+        <v>9</v>
+      </c>
+      <c r="E227" t="s">
         <v>614</v>
-      </c>
-      <c r="D227" t="s">
-        <v>9</v>
-      </c>
-      <c r="E227" t="s">
-        <v>615</v>
       </c>
       <c r="F227" t="s">
         <v>11</v>
@@ -7413,10 +7414,10 @@
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
+        <v>615</v>
+      </c>
+      <c r="B228" t="s">
         <v>616</v>
-      </c>
-      <c r="B228" t="s">
-        <v>617</v>
       </c>
       <c r="D228" t="s">
         <v>9</v>
@@ -7430,16 +7431,16 @@
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
+        <v>617</v>
+      </c>
+      <c r="B229" t="s">
         <v>618</v>
       </c>
-      <c r="B229" t="s">
+      <c r="D229" t="s">
+        <v>9</v>
+      </c>
+      <c r="E229" t="s">
         <v>619</v>
-      </c>
-      <c r="D229" t="s">
-        <v>9</v>
-      </c>
-      <c r="E229" t="s">
-        <v>620</v>
       </c>
       <c r="F229" t="s">
         <v>238</v>
@@ -7447,16 +7448,16 @@
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
+        <v>620</v>
+      </c>
+      <c r="B230" t="s">
         <v>621</v>
       </c>
-      <c r="B230" t="s">
+      <c r="D230" t="s">
+        <v>9</v>
+      </c>
+      <c r="E230" t="s">
         <v>622</v>
-      </c>
-      <c r="D230" t="s">
-        <v>9</v>
-      </c>
-      <c r="E230" t="s">
-        <v>623</v>
       </c>
       <c r="F230" t="s">
         <v>238</v>
@@ -7464,16 +7465,16 @@
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
+        <v>623</v>
+      </c>
+      <c r="B231" t="s">
         <v>624</v>
       </c>
-      <c r="B231" t="s">
+      <c r="D231" t="s">
+        <v>9</v>
+      </c>
+      <c r="E231" t="s">
         <v>625</v>
-      </c>
-      <c r="D231" t="s">
-        <v>9</v>
-      </c>
-      <c r="E231" t="s">
-        <v>626</v>
       </c>
       <c r="F231" t="s">
         <v>238</v>
@@ -7481,16 +7482,16 @@
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
+        <v>626</v>
+      </c>
+      <c r="B232" t="s">
         <v>627</v>
       </c>
-      <c r="B232" t="s">
+      <c r="D232" t="s">
+        <v>9</v>
+      </c>
+      <c r="E232" t="s">
         <v>628</v>
-      </c>
-      <c r="D232" t="s">
-        <v>9</v>
-      </c>
-      <c r="E232" t="s">
-        <v>629</v>
       </c>
       <c r="F232" t="s">
         <v>11</v>
@@ -7498,10 +7499,10 @@
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
+        <v>629</v>
+      </c>
+      <c r="B233" t="s">
         <v>630</v>
-      </c>
-      <c r="B233" t="s">
-        <v>631</v>
       </c>
       <c r="D233" t="s">
         <v>9</v>
@@ -7515,10 +7516,10 @@
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
+        <v>631</v>
+      </c>
+      <c r="B234" t="s">
         <v>632</v>
-      </c>
-      <c r="B234" t="s">
-        <v>633</v>
       </c>
       <c r="C234">
         <v>201</v>
@@ -7527,27 +7528,27 @@
         <v>43</v>
       </c>
       <c r="E234" t="s">
+        <v>633</v>
+      </c>
+      <c r="F234" t="s">
+        <v>238</v>
+      </c>
+      <c r="G234" t="s">
         <v>634</v>
-      </c>
-      <c r="F234" t="s">
-        <v>238</v>
-      </c>
-      <c r="G234" t="s">
-        <v>635</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
+        <v>635</v>
+      </c>
+      <c r="B235" t="s">
         <v>636</v>
       </c>
-      <c r="B235" t="s">
+      <c r="D235" t="s">
+        <v>9</v>
+      </c>
+      <c r="E235" t="s">
         <v>637</v>
-      </c>
-      <c r="D235" t="s">
-        <v>9</v>
-      </c>
-      <c r="E235" t="s">
-        <v>638</v>
       </c>
       <c r="F235" t="s">
         <v>238</v>
@@ -7555,16 +7556,16 @@
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
+        <v>638</v>
+      </c>
+      <c r="B236" t="s">
         <v>639</v>
       </c>
-      <c r="B236" t="s">
+      <c r="D236" t="s">
+        <v>9</v>
+      </c>
+      <c r="E236" t="s">
         <v>640</v>
-      </c>
-      <c r="D236" t="s">
-        <v>9</v>
-      </c>
-      <c r="E236" t="s">
-        <v>641</v>
       </c>
       <c r="F236" t="s">
         <v>11</v>
@@ -7572,16 +7573,16 @@
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
+        <v>641</v>
+      </c>
+      <c r="B237" t="s">
         <v>642</v>
       </c>
-      <c r="B237" t="s">
+      <c r="D237" t="s">
+        <v>9</v>
+      </c>
+      <c r="E237" t="s">
         <v>643</v>
-      </c>
-      <c r="D237" t="s">
-        <v>9</v>
-      </c>
-      <c r="E237" t="s">
-        <v>644</v>
       </c>
       <c r="F237" t="s">
         <v>238</v>
@@ -7589,16 +7590,16 @@
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
+        <v>644</v>
+      </c>
+      <c r="B238" t="s">
         <v>645</v>
       </c>
-      <c r="B238" t="s">
+      <c r="D238" t="s">
+        <v>9</v>
+      </c>
+      <c r="E238" t="s">
         <v>646</v>
-      </c>
-      <c r="D238" t="s">
-        <v>9</v>
-      </c>
-      <c r="E238" t="s">
-        <v>647</v>
       </c>
       <c r="F238" t="s">
         <v>11</v>
@@ -7606,16 +7607,16 @@
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
+        <v>647</v>
+      </c>
+      <c r="B239" t="s">
         <v>648</v>
       </c>
-      <c r="B239" t="s">
+      <c r="D239" t="s">
+        <v>9</v>
+      </c>
+      <c r="E239" t="s">
         <v>649</v>
-      </c>
-      <c r="D239" t="s">
-        <v>9</v>
-      </c>
-      <c r="E239" t="s">
-        <v>650</v>
       </c>
       <c r="F239" t="s">
         <v>11</v>
@@ -7623,10 +7624,10 @@
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
+        <v>650</v>
+      </c>
+      <c r="B240" t="s">
         <v>651</v>
-      </c>
-      <c r="B240" t="s">
-        <v>652</v>
       </c>
       <c r="D240" t="s">
         <v>9</v>
@@ -7640,10 +7641,10 @@
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
+        <v>652</v>
+      </c>
+      <c r="B241" t="s">
         <v>653</v>
-      </c>
-      <c r="B241" t="s">
-        <v>654</v>
       </c>
       <c r="D241" t="s">
         <v>9</v>
@@ -7657,10 +7658,10 @@
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
+        <v>654</v>
+      </c>
+      <c r="B242" t="s">
         <v>655</v>
-      </c>
-      <c r="B242" t="s">
-        <v>656</v>
       </c>
       <c r="D242" t="s">
         <v>9</v>
@@ -7674,16 +7675,16 @@
     </row>
     <row r="243" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
+        <v>656</v>
+      </c>
+      <c r="B243" t="s">
         <v>657</v>
       </c>
-      <c r="B243" t="s">
+      <c r="D243" t="s">
+        <v>9</v>
+      </c>
+      <c r="E243" t="s">
         <v>658</v>
-      </c>
-      <c r="D243" t="s">
-        <v>9</v>
-      </c>
-      <c r="E243" t="s">
-        <v>659</v>
       </c>
       <c r="F243" t="s">
         <v>238</v>
@@ -7691,16 +7692,16 @@
     </row>
     <row r="244" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
+        <v>659</v>
+      </c>
+      <c r="B244" t="s">
         <v>660</v>
       </c>
-      <c r="B244" t="s">
+      <c r="D244" t="s">
+        <v>9</v>
+      </c>
+      <c r="E244" t="s">
         <v>661</v>
-      </c>
-      <c r="D244" t="s">
-        <v>9</v>
-      </c>
-      <c r="E244" t="s">
-        <v>662</v>
       </c>
       <c r="F244" t="s">
         <v>238</v>
@@ -7708,7 +7709,7 @@
     </row>
     <row r="245" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
-        <v>663</v>
+        <v>662</v>
       </c>
       <c r="B245" t="s">
         <v>290</v>
@@ -7717,7 +7718,7 @@
         <v>9</v>
       </c>
       <c r="E245" t="s">
-        <v>664</v>
+        <v>663</v>
       </c>
       <c r="F245" t="s">
         <v>238</v>
@@ -7725,10 +7726,10 @@
     </row>
     <row r="246" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
+        <v>664</v>
+      </c>
+      <c r="B246" t="s">
         <v>665</v>
-      </c>
-      <c r="B246" t="s">
-        <v>666</v>
       </c>
       <c r="C246">
         <v>228</v>
@@ -7737,7 +7738,7 @@
         <v>21</v>
       </c>
       <c r="E246" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="F246" t="s">
         <v>238</v>
@@ -7745,16 +7746,16 @@
     </row>
     <row r="247" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
+        <v>667</v>
+      </c>
+      <c r="B247" t="s">
         <v>668</v>
       </c>
-      <c r="B247" t="s">
+      <c r="D247" t="s">
+        <v>9</v>
+      </c>
+      <c r="E247" t="s">
         <v>669</v>
-      </c>
-      <c r="D247" t="s">
-        <v>9</v>
-      </c>
-      <c r="E247" t="s">
-        <v>670</v>
       </c>
       <c r="F247" t="s">
         <v>238</v>
@@ -7762,16 +7763,16 @@
     </row>
     <row r="248" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
+        <v>670</v>
+      </c>
+      <c r="B248" t="s">
         <v>671</v>
       </c>
-      <c r="B248" t="s">
+      <c r="D248" t="s">
+        <v>9</v>
+      </c>
+      <c r="E248" t="s">
         <v>672</v>
-      </c>
-      <c r="D248" t="s">
-        <v>9</v>
-      </c>
-      <c r="E248" t="s">
-        <v>673</v>
       </c>
       <c r="F248" t="s">
         <v>238</v>
@@ -7779,16 +7780,16 @@
     </row>
     <row r="249" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
+        <v>673</v>
+      </c>
+      <c r="B249" t="s">
         <v>674</v>
       </c>
-      <c r="B249" t="s">
+      <c r="D249" t="s">
+        <v>9</v>
+      </c>
+      <c r="E249" t="s">
         <v>675</v>
-      </c>
-      <c r="D249" t="s">
-        <v>9</v>
-      </c>
-      <c r="E249" t="s">
-        <v>676</v>
       </c>
       <c r="F249" t="s">
         <v>238</v>
@@ -7796,30 +7797,30 @@
     </row>
     <row r="250" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
+        <v>676</v>
+      </c>
+      <c r="B250" t="s">
         <v>677</v>
       </c>
-      <c r="B250" t="s">
+      <c r="D250" t="s">
+        <v>9</v>
+      </c>
+      <c r="E250" t="s">
         <v>678</v>
       </c>
-      <c r="D250" t="s">
-        <v>9</v>
-      </c>
-      <c r="E250" t="s">
+      <c r="F250" t="s">
+        <v>11</v>
+      </c>
+      <c r="G250" t="s">
         <v>679</v>
-      </c>
-      <c r="F250" t="s">
-        <v>11</v>
-      </c>
-      <c r="G250" t="s">
-        <v>680</v>
       </c>
     </row>
     <row r="251" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
+        <v>680</v>
+      </c>
+      <c r="B251" t="s">
         <v>681</v>
-      </c>
-      <c r="B251" t="s">
-        <v>682</v>
       </c>
       <c r="C251">
         <v>207</v>
@@ -7828,7 +7829,7 @@
         <v>53</v>
       </c>
       <c r="E251" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="F251" t="s">
         <v>238</v>
@@ -7836,16 +7837,16 @@
     </row>
     <row r="252" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
+        <v>683</v>
+      </c>
+      <c r="B252" t="s">
         <v>684</v>
-      </c>
-      <c r="B252" t="s">
-        <v>685</v>
       </c>
       <c r="D252" t="s">
         <v>17</v>
       </c>
       <c r="E252" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
       <c r="F252" t="s">
         <v>238</v>
@@ -7853,10 +7854,10 @@
     </row>
     <row r="253" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
+        <v>686</v>
+      </c>
+      <c r="B253" t="s">
         <v>687</v>
-      </c>
-      <c r="B253" t="s">
-        <v>688</v>
       </c>
       <c r="C253">
         <v>211</v>
@@ -7865,7 +7866,7 @@
         <v>17</v>
       </c>
       <c r="E253" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
       <c r="F253" t="s">
         <v>238</v>
@@ -7873,16 +7874,16 @@
     </row>
     <row r="254" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
+        <v>689</v>
+      </c>
+      <c r="B254" t="s">
         <v>690</v>
       </c>
-      <c r="B254" t="s">
+      <c r="D254" t="s">
+        <v>9</v>
+      </c>
+      <c r="E254" t="s">
         <v>691</v>
-      </c>
-      <c r="D254" t="s">
-        <v>9</v>
-      </c>
-      <c r="E254" t="s">
-        <v>692</v>
       </c>
       <c r="F254" t="s">
         <v>238</v>
@@ -7890,16 +7891,16 @@
     </row>
     <row r="255" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
+        <v>692</v>
+      </c>
+      <c r="B255" t="s">
         <v>693</v>
-      </c>
-      <c r="B255" t="s">
-        <v>694</v>
       </c>
       <c r="D255" t="s">
         <v>53</v>
       </c>
       <c r="E255" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="F255" t="s">
         <v>238</v>
@@ -7907,16 +7908,16 @@
     </row>
     <row r="256" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
+        <v>695</v>
+      </c>
+      <c r="B256" t="s">
         <v>696</v>
       </c>
-      <c r="B256" t="s">
+      <c r="D256" t="s">
+        <v>9</v>
+      </c>
+      <c r="E256" t="s">
         <v>697</v>
-      </c>
-      <c r="D256" t="s">
-        <v>9</v>
-      </c>
-      <c r="E256" t="s">
-        <v>698</v>
       </c>
       <c r="F256" t="s">
         <v>238</v>
@@ -7924,10 +7925,10 @@
     </row>
     <row r="257" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
+        <v>698</v>
+      </c>
+      <c r="B257" t="s">
         <v>699</v>
-      </c>
-      <c r="B257" t="s">
-        <v>700</v>
       </c>
       <c r="C257">
         <v>230</v>
@@ -7936,7 +7937,7 @@
         <v>53</v>
       </c>
       <c r="E257" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="F257" t="s">
         <v>238</v>
@@ -7944,16 +7945,16 @@
     </row>
     <row r="258" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
+        <v>701</v>
+      </c>
+      <c r="B258" t="s">
         <v>702</v>
       </c>
-      <c r="B258" t="s">
+      <c r="D258" t="s">
+        <v>9</v>
+      </c>
+      <c r="E258" t="s">
         <v>703</v>
-      </c>
-      <c r="D258" t="s">
-        <v>9</v>
-      </c>
-      <c r="E258" t="s">
-        <v>704</v>
       </c>
       <c r="F258" t="s">
         <v>238</v>
@@ -7961,16 +7962,16 @@
     </row>
     <row r="259" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
+        <v>704</v>
+      </c>
+      <c r="B259" t="s">
         <v>705</v>
       </c>
-      <c r="B259" t="s">
+      <c r="D259" t="s">
+        <v>9</v>
+      </c>
+      <c r="E259" t="s">
         <v>706</v>
-      </c>
-      <c r="D259" t="s">
-        <v>9</v>
-      </c>
-      <c r="E259" t="s">
-        <v>707</v>
       </c>
       <c r="F259" t="s">
         <v>238</v>
@@ -7978,16 +7979,16 @@
     </row>
     <row r="260" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
+        <v>707</v>
+      </c>
+      <c r="B260" t="s">
         <v>708</v>
       </c>
-      <c r="B260" t="s">
+      <c r="D260" t="s">
+        <v>9</v>
+      </c>
+      <c r="E260" t="s">
         <v>709</v>
-      </c>
-      <c r="D260" t="s">
-        <v>9</v>
-      </c>
-      <c r="E260" t="s">
-        <v>710</v>
       </c>
       <c r="F260" t="s">
         <v>238</v>
@@ -7995,16 +7996,16 @@
     </row>
     <row r="261" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
+        <v>710</v>
+      </c>
+      <c r="B261" t="s">
         <v>711</v>
       </c>
-      <c r="B261" t="s">
+      <c r="D261" t="s">
+        <v>9</v>
+      </c>
+      <c r="E261" t="s">
         <v>712</v>
-      </c>
-      <c r="D261" t="s">
-        <v>9</v>
-      </c>
-      <c r="E261" t="s">
-        <v>713</v>
       </c>
       <c r="F261" t="s">
         <v>238</v>
@@ -8012,16 +8013,16 @@
     </row>
     <row r="262" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
+        <v>713</v>
+      </c>
+      <c r="B262" t="s">
         <v>714</v>
       </c>
-      <c r="B262" t="s">
+      <c r="D262" t="s">
+        <v>9</v>
+      </c>
+      <c r="E262" t="s">
         <v>715</v>
-      </c>
-      <c r="D262" t="s">
-        <v>9</v>
-      </c>
-      <c r="E262" t="s">
-        <v>716</v>
       </c>
       <c r="F262" t="s">
         <v>238</v>
@@ -8029,16 +8030,16 @@
     </row>
     <row r="263" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
+        <v>716</v>
+      </c>
+      <c r="B263" t="s">
         <v>717</v>
       </c>
-      <c r="B263" t="s">
+      <c r="D263" t="s">
+        <v>9</v>
+      </c>
+      <c r="E263" t="s">
         <v>718</v>
-      </c>
-      <c r="D263" t="s">
-        <v>9</v>
-      </c>
-      <c r="E263" t="s">
-        <v>719</v>
       </c>
       <c r="F263" t="s">
         <v>238</v>
@@ -8046,16 +8047,16 @@
     </row>
     <row r="264" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
+        <v>719</v>
+      </c>
+      <c r="B264" t="s">
         <v>720</v>
       </c>
-      <c r="B264" t="s">
+      <c r="D264" t="s">
+        <v>9</v>
+      </c>
+      <c r="E264" t="s">
         <v>721</v>
-      </c>
-      <c r="D264" t="s">
-        <v>9</v>
-      </c>
-      <c r="E264" t="s">
-        <v>722</v>
       </c>
       <c r="F264" t="s">
         <v>238</v>
@@ -8063,10 +8064,10 @@
     </row>
     <row r="265" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
+        <v>722</v>
+      </c>
+      <c r="B265" t="s">
         <v>723</v>
-      </c>
-      <c r="B265" t="s">
-        <v>724</v>
       </c>
       <c r="D265" t="s">
         <v>9</v>
@@ -8080,16 +8081,16 @@
     </row>
     <row r="266" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
+        <v>724</v>
+      </c>
+      <c r="B266" t="s">
         <v>725</v>
       </c>
-      <c r="B266" t="s">
+      <c r="D266" t="s">
+        <v>9</v>
+      </c>
+      <c r="E266" t="s">
         <v>726</v>
-      </c>
-      <c r="D266" t="s">
-        <v>9</v>
-      </c>
-      <c r="E266" t="s">
-        <v>727</v>
       </c>
       <c r="F266" t="s">
         <v>238</v>
@@ -8097,16 +8098,16 @@
     </row>
     <row r="267" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
+        <v>727</v>
+      </c>
+      <c r="B267" t="s">
         <v>728</v>
-      </c>
-      <c r="B267" t="s">
-        <v>729</v>
       </c>
       <c r="D267" t="s">
         <v>17</v>
       </c>
       <c r="E267" t="s">
-        <v>730</v>
+        <v>729</v>
       </c>
       <c r="F267" t="s">
         <v>238</v>
@@ -8114,16 +8115,16 @@
     </row>
     <row r="268" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
+        <v>730</v>
+      </c>
+      <c r="B268" t="s">
         <v>731</v>
       </c>
-      <c r="B268" t="s">
+      <c r="D268" t="s">
+        <v>9</v>
+      </c>
+      <c r="E268" t="s">
         <v>732</v>
-      </c>
-      <c r="D268" t="s">
-        <v>9</v>
-      </c>
-      <c r="E268" t="s">
-        <v>733</v>
       </c>
       <c r="F268" t="s">
         <v>238</v>
@@ -8131,36 +8132,36 @@
     </row>
     <row r="269" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
+        <v>733</v>
+      </c>
+      <c r="B269" t="s">
         <v>734</v>
       </c>
-      <c r="B269" t="s">
+      <c r="D269" t="s">
+        <v>9</v>
+      </c>
+      <c r="E269" t="s">
         <v>735</v>
       </c>
-      <c r="D269" t="s">
-        <v>9</v>
-      </c>
-      <c r="E269" t="s">
+      <c r="F269" t="s">
+        <v>238</v>
+      </c>
+      <c r="G269" t="s">
         <v>736</v>
-      </c>
-      <c r="F269" t="s">
-        <v>238</v>
-      </c>
-      <c r="G269" t="s">
-        <v>737</v>
       </c>
     </row>
     <row r="270" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
+        <v>737</v>
+      </c>
+      <c r="B270" t="s">
         <v>738</v>
       </c>
-      <c r="B270" t="s">
+      <c r="D270" t="s">
+        <v>9</v>
+      </c>
+      <c r="E270" t="s">
         <v>739</v>
-      </c>
-      <c r="D270" t="s">
-        <v>9</v>
-      </c>
-      <c r="E270" t="s">
-        <v>740</v>
       </c>
       <c r="F270" t="s">
         <v>238</v>
@@ -8168,36 +8169,36 @@
     </row>
     <row r="271" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A271" t="s">
+        <v>740</v>
+      </c>
+      <c r="B271" t="s">
         <v>741</v>
       </c>
-      <c r="B271" t="s">
+      <c r="D271" t="s">
+        <v>9</v>
+      </c>
+      <c r="E271" t="s">
         <v>742</v>
       </c>
-      <c r="D271" t="s">
-        <v>9</v>
-      </c>
-      <c r="E271" t="s">
+      <c r="F271" t="s">
+        <v>238</v>
+      </c>
+      <c r="G271" t="s">
         <v>743</v>
-      </c>
-      <c r="F271" t="s">
-        <v>238</v>
-      </c>
-      <c r="G271" t="s">
-        <v>744</v>
       </c>
     </row>
     <row r="272" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A272" t="s">
+        <v>744</v>
+      </c>
+      <c r="B272" t="s">
         <v>745</v>
       </c>
-      <c r="B272" t="s">
+      <c r="D272" t="s">
+        <v>9</v>
+      </c>
+      <c r="E272" t="s">
         <v>746</v>
-      </c>
-      <c r="D272" t="s">
-        <v>9</v>
-      </c>
-      <c r="E272" t="s">
-        <v>747</v>
       </c>
       <c r="F272" t="s">
         <v>238</v>
@@ -8205,10 +8206,10 @@
     </row>
     <row r="273" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A273" t="s">
+        <v>747</v>
+      </c>
+      <c r="B273" t="s">
         <v>748</v>
-      </c>
-      <c r="B273" t="s">
-        <v>749</v>
       </c>
       <c r="C273">
         <v>220</v>
@@ -8225,16 +8226,16 @@
     </row>
     <row r="274" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A274" t="s">
+        <v>749</v>
+      </c>
+      <c r="B274" t="s">
         <v>750</v>
       </c>
-      <c r="B274" t="s">
+      <c r="D274" t="s">
+        <v>9</v>
+      </c>
+      <c r="E274" t="s">
         <v>751</v>
-      </c>
-      <c r="D274" t="s">
-        <v>9</v>
-      </c>
-      <c r="E274" t="s">
-        <v>752</v>
       </c>
       <c r="F274" t="s">
         <v>11</v>
@@ -8242,16 +8243,16 @@
     </row>
     <row r="275" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A275" t="s">
+        <v>752</v>
+      </c>
+      <c r="B275" t="s">
         <v>753</v>
       </c>
-      <c r="B275" t="s">
+      <c r="D275" t="s">
+        <v>9</v>
+      </c>
+      <c r="E275" t="s">
         <v>754</v>
-      </c>
-      <c r="D275" t="s">
-        <v>9</v>
-      </c>
-      <c r="E275" t="s">
-        <v>755</v>
       </c>
       <c r="F275" t="s">
         <v>238</v>
@@ -8259,10 +8260,10 @@
     </row>
     <row r="276" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A276" t="s">
+        <v>755</v>
+      </c>
+      <c r="B276" t="s">
         <v>756</v>
-      </c>
-      <c r="B276" t="s">
-        <v>757</v>
       </c>
       <c r="C276">
         <v>196</v>
@@ -8271,27 +8272,27 @@
         <v>17</v>
       </c>
       <c r="E276" t="s">
+        <v>757</v>
+      </c>
+      <c r="F276" t="s">
+        <v>238</v>
+      </c>
+      <c r="G276" t="s">
         <v>758</v>
-      </c>
-      <c r="F276" t="s">
-        <v>238</v>
-      </c>
-      <c r="G276" t="s">
-        <v>759</v>
       </c>
     </row>
     <row r="277" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A277" t="s">
+        <v>759</v>
+      </c>
+      <c r="B277" t="s">
         <v>760</v>
       </c>
-      <c r="B277" t="s">
+      <c r="D277" t="s">
+        <v>9</v>
+      </c>
+      <c r="E277" t="s">
         <v>761</v>
-      </c>
-      <c r="D277" t="s">
-        <v>9</v>
-      </c>
-      <c r="E277" t="s">
-        <v>762</v>
       </c>
       <c r="F277" t="s">
         <v>238</v>
@@ -8299,16 +8300,16 @@
     </row>
     <row r="278" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A278" t="s">
+        <v>762</v>
+      </c>
+      <c r="B278" t="s">
         <v>763</v>
       </c>
-      <c r="B278" t="s">
+      <c r="D278" t="s">
+        <v>9</v>
+      </c>
+      <c r="E278" t="s">
         <v>764</v>
-      </c>
-      <c r="D278" t="s">
-        <v>9</v>
-      </c>
-      <c r="E278" t="s">
-        <v>765</v>
       </c>
       <c r="F278" t="s">
         <v>238</v>
@@ -8316,30 +8317,30 @@
     </row>
     <row r="279" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A279" t="s">
+        <v>765</v>
+      </c>
+      <c r="B279" t="s">
         <v>766</v>
-      </c>
-      <c r="B279" t="s">
-        <v>767</v>
       </c>
       <c r="D279" t="s">
         <v>21</v>
       </c>
       <c r="E279" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="F279" t="s">
         <v>238</v>
       </c>
       <c r="G279" t="s">
-        <v>824</v>
+        <v>823</v>
       </c>
     </row>
     <row r="280" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A280" t="s">
+        <v>768</v>
+      </c>
+      <c r="B280" t="s">
         <v>769</v>
-      </c>
-      <c r="B280" t="s">
-        <v>770</v>
       </c>
       <c r="D280" t="s">
         <v>9</v>
@@ -8353,16 +8354,16 @@
     </row>
     <row r="281" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A281" t="s">
+        <v>770</v>
+      </c>
+      <c r="B281" t="s">
         <v>771</v>
       </c>
-      <c r="B281" t="s">
+      <c r="D281" t="s">
+        <v>9</v>
+      </c>
+      <c r="E281" t="s">
         <v>772</v>
-      </c>
-      <c r="D281" t="s">
-        <v>9</v>
-      </c>
-      <c r="E281" t="s">
-        <v>773</v>
       </c>
       <c r="F281" t="s">
         <v>11</v>
@@ -8370,16 +8371,16 @@
     </row>
     <row r="282" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A282" t="s">
+        <v>773</v>
+      </c>
+      <c r="B282" t="s">
         <v>774</v>
-      </c>
-      <c r="B282" t="s">
-        <v>775</v>
       </c>
       <c r="D282" t="s">
         <v>17</v>
       </c>
       <c r="E282" t="s">
-        <v>776</v>
+        <v>775</v>
       </c>
       <c r="F282" t="s">
         <v>238</v>
@@ -8387,16 +8388,16 @@
     </row>
     <row r="283" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A283" t="s">
+        <v>776</v>
+      </c>
+      <c r="B283" t="s">
         <v>777</v>
       </c>
-      <c r="B283" t="s">
+      <c r="D283" t="s">
+        <v>9</v>
+      </c>
+      <c r="E283" t="s">
         <v>778</v>
-      </c>
-      <c r="D283" t="s">
-        <v>9</v>
-      </c>
-      <c r="E283" t="s">
-        <v>779</v>
       </c>
       <c r="F283" t="s">
         <v>238</v>
@@ -8404,16 +8405,16 @@
     </row>
     <row r="284" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A284" t="s">
+        <v>779</v>
+      </c>
+      <c r="B284" t="s">
         <v>780</v>
       </c>
-      <c r="B284" t="s">
+      <c r="D284" t="s">
+        <v>9</v>
+      </c>
+      <c r="E284" t="s">
         <v>781</v>
-      </c>
-      <c r="D284" t="s">
-        <v>9</v>
-      </c>
-      <c r="E284" t="s">
-        <v>782</v>
       </c>
       <c r="F284" t="s">
         <v>238</v>
@@ -8421,10 +8422,10 @@
     </row>
     <row r="285" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A285" t="s">
+        <v>782</v>
+      </c>
+      <c r="B285" t="s">
         <v>783</v>
-      </c>
-      <c r="B285" t="s">
-        <v>784</v>
       </c>
       <c r="D285" t="s">
         <v>17</v>
@@ -8438,16 +8439,16 @@
     </row>
     <row r="286" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A286" t="s">
+        <v>784</v>
+      </c>
+      <c r="B286" t="s">
         <v>785</v>
       </c>
-      <c r="B286" t="s">
+      <c r="D286" t="s">
+        <v>9</v>
+      </c>
+      <c r="E286" t="s">
         <v>786</v>
-      </c>
-      <c r="D286" t="s">
-        <v>9</v>
-      </c>
-      <c r="E286" t="s">
-        <v>787</v>
       </c>
       <c r="F286" t="s">
         <v>238</v>
@@ -8455,16 +8456,16 @@
     </row>
     <row r="287" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A287" t="s">
+        <v>787</v>
+      </c>
+      <c r="B287" t="s">
         <v>788</v>
       </c>
-      <c r="B287" t="s">
+      <c r="D287" t="s">
+        <v>9</v>
+      </c>
+      <c r="E287" t="s">
         <v>789</v>
-      </c>
-      <c r="D287" t="s">
-        <v>9</v>
-      </c>
-      <c r="E287" t="s">
-        <v>790</v>
       </c>
       <c r="F287" t="s">
         <v>238</v>
@@ -8472,7 +8473,7 @@
     </row>
     <row r="288" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A288" t="s">
-        <v>791</v>
+        <v>790</v>
       </c>
       <c r="B288" t="s">
         <v>167</v>
@@ -8481,7 +8482,7 @@
         <v>17</v>
       </c>
       <c r="E288" t="s">
-        <v>792</v>
+        <v>791</v>
       </c>
       <c r="F288" t="s">
         <v>238</v>
@@ -8489,16 +8490,16 @@
     </row>
     <row r="289" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A289" t="s">
+        <v>792</v>
+      </c>
+      <c r="B289" t="s">
         <v>793</v>
       </c>
-      <c r="B289" t="s">
+      <c r="D289" t="s">
+        <v>9</v>
+      </c>
+      <c r="E289" t="s">
         <v>794</v>
-      </c>
-      <c r="D289" t="s">
-        <v>9</v>
-      </c>
-      <c r="E289" t="s">
-        <v>795</v>
       </c>
       <c r="F289" t="s">
         <v>238</v>
@@ -8506,16 +8507,16 @@
     </row>
     <row r="290" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A290" t="s">
+        <v>795</v>
+      </c>
+      <c r="B290" t="s">
         <v>796</v>
       </c>
-      <c r="B290" t="s">
+      <c r="D290" t="s">
+        <v>9</v>
+      </c>
+      <c r="E290" t="s">
         <v>797</v>
-      </c>
-      <c r="D290" t="s">
-        <v>9</v>
-      </c>
-      <c r="E290" t="s">
-        <v>798</v>
       </c>
       <c r="F290" t="s">
         <v>238</v>
@@ -8523,16 +8524,16 @@
     </row>
     <row r="291" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A291" t="s">
+        <v>798</v>
+      </c>
+      <c r="B291" t="s">
         <v>799</v>
       </c>
-      <c r="B291" t="s">
+      <c r="D291" t="s">
+        <v>9</v>
+      </c>
+      <c r="E291" t="s">
         <v>800</v>
-      </c>
-      <c r="D291" t="s">
-        <v>9</v>
-      </c>
-      <c r="E291" t="s">
-        <v>801</v>
       </c>
       <c r="F291" t="s">
         <v>238</v>
@@ -8540,16 +8541,16 @@
     </row>
     <row r="292" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A292" t="s">
+        <v>801</v>
+      </c>
+      <c r="B292" t="s">
         <v>802</v>
       </c>
-      <c r="B292" t="s">
+      <c r="D292" t="s">
+        <v>9</v>
+      </c>
+      <c r="E292" t="s">
         <v>803</v>
-      </c>
-      <c r="D292" t="s">
-        <v>9</v>
-      </c>
-      <c r="E292" t="s">
-        <v>804</v>
       </c>
       <c r="F292" t="s">
         <v>238</v>
@@ -8557,16 +8558,16 @@
     </row>
     <row r="293" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A293" t="s">
+        <v>804</v>
+      </c>
+      <c r="B293" t="s">
         <v>805</v>
       </c>
-      <c r="B293" t="s">
+      <c r="D293" t="s">
+        <v>9</v>
+      </c>
+      <c r="E293" t="s">
         <v>806</v>
-      </c>
-      <c r="D293" t="s">
-        <v>9</v>
-      </c>
-      <c r="E293" t="s">
-        <v>807</v>
       </c>
       <c r="F293" t="s">
         <v>238</v>
@@ -8574,10 +8575,10 @@
     </row>
     <row r="294" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A294" t="s">
+        <v>807</v>
+      </c>
+      <c r="B294" t="s">
         <v>808</v>
-      </c>
-      <c r="B294" t="s">
-        <v>809</v>
       </c>
       <c r="D294" t="s">
         <v>17</v>
@@ -8591,10 +8592,10 @@
     </row>
     <row r="295" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A295" t="s">
-        <v>825</v>
+        <v>824</v>
       </c>
       <c r="B295" t="s">
-        <v>810</v>
+        <v>809</v>
       </c>
       <c r="D295" t="s">
         <v>17</v>
@@ -8608,10 +8609,10 @@
     </row>
     <row r="296" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A296" t="s">
+        <v>810</v>
+      </c>
+      <c r="B296" t="s">
         <v>811</v>
-      </c>
-      <c r="B296" t="s">
-        <v>812</v>
       </c>
       <c r="D296" t="s">
         <v>17</v>
@@ -8625,10 +8626,10 @@
     </row>
     <row r="297" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A297" t="s">
+        <v>812</v>
+      </c>
+      <c r="B297" t="s">
         <v>813</v>
-      </c>
-      <c r="B297" t="s">
-        <v>814</v>
       </c>
       <c r="D297" t="s">
         <v>17</v>
@@ -8642,10 +8643,10 @@
     </row>
     <row r="298" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A298" t="s">
+        <v>814</v>
+      </c>
+      <c r="B298" t="s">
         <v>815</v>
-      </c>
-      <c r="B298" t="s">
-        <v>816</v>
       </c>
       <c r="D298" t="s">
         <v>17</v>
@@ -8659,16 +8660,16 @@
     </row>
     <row r="299" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A299" t="s">
+        <v>816</v>
+      </c>
+      <c r="B299" t="s">
         <v>817</v>
-      </c>
-      <c r="B299" t="s">
-        <v>818</v>
       </c>
       <c r="D299" t="s">
         <v>37</v>
       </c>
       <c r="E299" t="s">
-        <v>819</v>
+        <v>818</v>
       </c>
       <c r="F299" t="s">
         <v>238</v>
@@ -8676,10 +8677,10 @@
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A300" t="s">
+        <v>819</v>
+      </c>
+      <c r="B300" t="s">
         <v>820</v>
-      </c>
-      <c r="B300" t="s">
-        <v>821</v>
       </c>
       <c r="D300" t="s">
         <v>37</v>
@@ -8693,10 +8694,10 @@
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A301" t="s">
+        <v>821</v>
+      </c>
+      <c r="B301" t="s">
         <v>822</v>
-      </c>
-      <c r="B301" t="s">
-        <v>823</v>
       </c>
       <c r="D301" t="s">
         <v>37</v>

</xml_diff>